<commit_message>
Fix generatePO bug, month_start_inv bug
</commit_message>
<xml_diff>
--- a/history_data/usage_history-temp.xlsx
+++ b/history_data/usage_history-temp.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:V58"/>
+  <dimension ref="A1:V96"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -553,11 +553,11 @@
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>2026-02-01~2026-02-28</t>
+          <t>2026-07-01~2026-07-31</t>
         </is>
       </c>
       <c r="D2" t="n">
-        <v>28</v>
+        <v>31</v>
       </c>
       <c r="E2" t="inlineStr">
         <is>
@@ -570,20 +570,20 @@
         </is>
       </c>
       <c r="G2" t="n">
-        <v>0</v>
+        <v>2755</v>
       </c>
       <c r="H2" t="inlineStr"/>
       <c r="I2" t="n">
         <v>0</v>
       </c>
       <c r="J2" t="n">
-        <v>0</v>
+        <v>2755</v>
       </c>
       <c r="K2" t="n">
         <v>1</v>
       </c>
       <c r="L2" t="n">
-        <v>0</v>
+        <v>2755</v>
       </c>
       <c r="M2" t="inlineStr"/>
       <c r="N2" t="inlineStr"/>
@@ -611,7 +611,7 @@
         <v>2000</v>
       </c>
       <c r="V2" t="n">
-        <v>0</v>
+        <v>2755</v>
       </c>
     </row>
     <row r="3">
@@ -627,11 +627,11 @@
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>2026-02-01~2026-02-28</t>
+          <t>2026-07-01~2026-07-31</t>
         </is>
       </c>
       <c r="D3" t="n">
-        <v>28</v>
+        <v>31</v>
       </c>
       <c r="E3" t="inlineStr">
         <is>
@@ -644,20 +644,20 @@
         </is>
       </c>
       <c r="G3" t="n">
-        <v>800</v>
+        <v>5479</v>
       </c>
       <c r="H3" t="inlineStr"/>
       <c r="I3" t="n">
         <v>0</v>
       </c>
       <c r="J3" t="n">
-        <v>800</v>
+        <v>5479</v>
       </c>
       <c r="K3" t="n">
         <v>1</v>
       </c>
       <c r="L3" t="n">
-        <v>800</v>
+        <v>5479</v>
       </c>
       <c r="M3" t="inlineStr"/>
       <c r="N3" t="inlineStr"/>
@@ -685,7 +685,7 @@
         <v>1000</v>
       </c>
       <c r="V3" t="n">
-        <v>800</v>
+        <v>5479</v>
       </c>
     </row>
     <row r="4">
@@ -701,11 +701,11 @@
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>2026-02-01~2026-02-28</t>
+          <t>2026-07-01~2026-07-31</t>
         </is>
       </c>
       <c r="D4" t="n">
-        <v>28</v>
+        <v>31</v>
       </c>
       <c r="E4" t="inlineStr">
         <is>
@@ -718,20 +718,20 @@
         </is>
       </c>
       <c r="G4" t="n">
-        <v>2050</v>
+        <v>21877</v>
       </c>
       <c r="H4" t="inlineStr"/>
       <c r="I4" t="n">
         <v>0</v>
       </c>
       <c r="J4" t="n">
-        <v>2050</v>
+        <v>21877</v>
       </c>
       <c r="K4" t="n">
         <v>1</v>
       </c>
       <c r="L4" t="n">
-        <v>2050</v>
+        <v>21877</v>
       </c>
       <c r="M4" t="inlineStr"/>
       <c r="N4" t="inlineStr"/>
@@ -759,7 +759,7 @@
         <v>500</v>
       </c>
       <c r="V4" t="n">
-        <v>61.5</v>
+        <v>656.3099999999999</v>
       </c>
     </row>
     <row r="5">
@@ -775,11 +775,11 @@
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>2026-02-01~2026-02-28</t>
+          <t>2026-07-01~2026-07-31</t>
         </is>
       </c>
       <c r="D5" t="n">
-        <v>28</v>
+        <v>31</v>
       </c>
       <c r="E5" t="inlineStr">
         <is>
@@ -792,20 +792,20 @@
         </is>
       </c>
       <c r="G5" t="n">
-        <v>1610</v>
+        <v>21097</v>
       </c>
       <c r="H5" t="inlineStr"/>
       <c r="I5" t="n">
         <v>0</v>
       </c>
       <c r="J5" t="n">
-        <v>1610</v>
+        <v>21097</v>
       </c>
       <c r="K5" t="n">
         <v>1</v>
       </c>
       <c r="L5" t="n">
-        <v>1610</v>
+        <v>21097</v>
       </c>
       <c r="M5" t="inlineStr"/>
       <c r="N5" t="inlineStr"/>
@@ -823,7 +823,7 @@
       <c r="T5" t="inlineStr"/>
       <c r="U5" t="inlineStr"/>
       <c r="V5" t="n">
-        <v>1610</v>
+        <v>21097</v>
       </c>
     </row>
     <row r="6">
@@ -839,11 +839,11 @@
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>2026-02-01~2026-02-28</t>
+          <t>2026-07-01~2026-07-31</t>
         </is>
       </c>
       <c r="D6" t="n">
-        <v>28</v>
+        <v>31</v>
       </c>
       <c r="E6" t="inlineStr">
         <is>
@@ -856,20 +856,20 @@
         </is>
       </c>
       <c r="G6" t="n">
-        <v>0</v>
+        <v>12315</v>
       </c>
       <c r="H6" t="inlineStr"/>
       <c r="I6" t="n">
         <v>0</v>
       </c>
       <c r="J6" t="n">
-        <v>0</v>
+        <v>12315</v>
       </c>
       <c r="K6" t="n">
         <v>1</v>
       </c>
       <c r="L6" t="n">
-        <v>0</v>
+        <v>12315</v>
       </c>
       <c r="M6" t="inlineStr"/>
       <c r="N6" t="inlineStr"/>
@@ -897,7 +897,7 @@
         <v>500</v>
       </c>
       <c r="V6" t="n">
-        <v>0</v>
+        <v>369.45</v>
       </c>
     </row>
     <row r="7">
@@ -913,11 +913,11 @@
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>2026-02-01~2026-02-28</t>
+          <t>2026-07-01~2026-07-31</t>
         </is>
       </c>
       <c r="D7" t="n">
-        <v>28</v>
+        <v>31</v>
       </c>
       <c r="E7" t="inlineStr">
         <is>
@@ -930,20 +930,20 @@
         </is>
       </c>
       <c r="G7" t="n">
-        <v>800</v>
+        <v>3571</v>
       </c>
       <c r="H7" t="inlineStr"/>
       <c r="I7" t="n">
         <v>0</v>
       </c>
       <c r="J7" t="n">
-        <v>800</v>
+        <v>3571</v>
       </c>
       <c r="K7" t="n">
         <v>1</v>
       </c>
       <c r="L7" t="n">
-        <v>800</v>
+        <v>3571</v>
       </c>
       <c r="M7" t="inlineStr"/>
       <c r="N7" t="inlineStr"/>
@@ -971,7 +971,7 @@
         <v>2000</v>
       </c>
       <c r="V7" t="n">
-        <v>800</v>
+        <v>3571</v>
       </c>
     </row>
     <row r="8">
@@ -987,11 +987,11 @@
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>2026-02-01~2026-02-28</t>
+          <t>2026-07-01~2026-07-31</t>
         </is>
       </c>
       <c r="D8" t="n">
-        <v>28</v>
+        <v>31</v>
       </c>
       <c r="E8" t="inlineStr">
         <is>
@@ -1004,20 +1004,20 @@
         </is>
       </c>
       <c r="G8" t="n">
-        <v>0</v>
+        <v>1345</v>
       </c>
       <c r="H8" t="inlineStr"/>
       <c r="I8" t="n">
         <v>0</v>
       </c>
       <c r="J8" t="n">
-        <v>0</v>
+        <v>1345</v>
       </c>
       <c r="K8" t="n">
         <v>1</v>
       </c>
       <c r="L8" t="n">
-        <v>0</v>
+        <v>1345</v>
       </c>
       <c r="M8" t="inlineStr"/>
       <c r="N8" t="inlineStr"/>
@@ -1045,7 +1045,7 @@
         <v>2000</v>
       </c>
       <c r="V8" t="n">
-        <v>0</v>
+        <v>1345</v>
       </c>
     </row>
     <row r="9">
@@ -1061,11 +1061,11 @@
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>2026-02-01~2026-02-28</t>
+          <t>2026-07-01~2026-07-31</t>
         </is>
       </c>
       <c r="D9" t="n">
-        <v>28</v>
+        <v>31</v>
       </c>
       <c r="E9" t="inlineStr">
         <is>
@@ -1125,11 +1125,11 @@
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>2026-02-01~2026-02-28</t>
+          <t>2026-07-01~2026-07-31</t>
         </is>
       </c>
       <c r="D10" t="n">
-        <v>28</v>
+        <v>31</v>
       </c>
       <c r="E10" t="inlineStr">
         <is>
@@ -1142,20 +1142,20 @@
         </is>
       </c>
       <c r="G10" t="n">
-        <v>0</v>
+        <v>3600</v>
       </c>
       <c r="H10" t="inlineStr"/>
       <c r="I10" t="n">
         <v>0</v>
       </c>
       <c r="J10" t="n">
-        <v>0</v>
+        <v>3600</v>
       </c>
       <c r="K10" t="n">
         <v>1</v>
       </c>
       <c r="L10" t="n">
-        <v>0</v>
+        <v>3600</v>
       </c>
       <c r="M10" t="inlineStr"/>
       <c r="N10" t="inlineStr"/>
@@ -1183,7 +1183,7 @@
         <v>2000</v>
       </c>
       <c r="V10" t="n">
-        <v>0</v>
+        <v>3600</v>
       </c>
     </row>
     <row r="11">
@@ -1199,11 +1199,11 @@
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>2026-02-01~2026-02-28</t>
+          <t>2026-07-01~2026-07-31</t>
         </is>
       </c>
       <c r="D11" t="n">
-        <v>28</v>
+        <v>31</v>
       </c>
       <c r="E11" t="inlineStr">
         <is>
@@ -1216,20 +1216,20 @@
         </is>
       </c>
       <c r="G11" t="n">
-        <v>150</v>
+        <v>0</v>
       </c>
       <c r="H11" t="inlineStr"/>
       <c r="I11" t="n">
         <v>0</v>
       </c>
       <c r="J11" t="n">
-        <v>150</v>
+        <v>0</v>
       </c>
       <c r="K11" t="n">
         <v>1</v>
       </c>
       <c r="L11" t="n">
-        <v>150</v>
+        <v>0</v>
       </c>
       <c r="M11" t="inlineStr"/>
       <c r="N11" t="inlineStr"/>
@@ -1247,7 +1247,7 @@
       <c r="T11" t="inlineStr"/>
       <c r="U11" t="inlineStr"/>
       <c r="V11" t="n">
-        <v>150</v>
+        <v>0</v>
       </c>
     </row>
     <row r="12">
@@ -1263,11 +1263,11 @@
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>2026-02-01~2026-02-28</t>
+          <t>2026-07-01~2026-07-31</t>
         </is>
       </c>
       <c r="D12" t="n">
-        <v>28</v>
+        <v>31</v>
       </c>
       <c r="E12" t="inlineStr">
         <is>
@@ -1280,20 +1280,20 @@
         </is>
       </c>
       <c r="G12" t="n">
-        <v>400</v>
+        <v>0</v>
       </c>
       <c r="H12" t="inlineStr"/>
       <c r="I12" t="n">
         <v>0</v>
       </c>
       <c r="J12" t="n">
-        <v>400</v>
+        <v>0</v>
       </c>
       <c r="K12" t="n">
         <v>1</v>
       </c>
       <c r="L12" t="n">
-        <v>400</v>
+        <v>0</v>
       </c>
       <c r="M12" t="inlineStr"/>
       <c r="N12" t="inlineStr"/>
@@ -1311,7 +1311,7 @@
       <c r="T12" t="inlineStr"/>
       <c r="U12" t="inlineStr"/>
       <c r="V12" t="n">
-        <v>400</v>
+        <v>0</v>
       </c>
     </row>
     <row r="13">
@@ -1327,11 +1327,11 @@
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>2026-02-01~2026-02-28</t>
+          <t>2026-07-01~2026-07-31</t>
         </is>
       </c>
       <c r="D13" t="n">
-        <v>28</v>
+        <v>31</v>
       </c>
       <c r="E13" t="inlineStr">
         <is>
@@ -1344,20 +1344,20 @@
         </is>
       </c>
       <c r="G13" t="n">
-        <v>150</v>
+        <v>0</v>
       </c>
       <c r="H13" t="inlineStr"/>
       <c r="I13" t="n">
         <v>0</v>
       </c>
       <c r="J13" t="n">
-        <v>150</v>
+        <v>0</v>
       </c>
       <c r="K13" t="n">
         <v>1</v>
       </c>
       <c r="L13" t="n">
-        <v>150</v>
+        <v>0</v>
       </c>
       <c r="M13" t="inlineStr"/>
       <c r="N13" t="inlineStr"/>
@@ -1375,7 +1375,7 @@
       <c r="T13" t="inlineStr"/>
       <c r="U13" t="inlineStr"/>
       <c r="V13" t="n">
-        <v>150</v>
+        <v>0</v>
       </c>
     </row>
     <row r="14">
@@ -1391,11 +1391,11 @@
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>2026-02-01~2026-02-28</t>
+          <t>2026-07-01~2026-07-31</t>
         </is>
       </c>
       <c r="D14" t="n">
-        <v>28</v>
+        <v>31</v>
       </c>
       <c r="E14" t="inlineStr">
         <is>
@@ -1455,11 +1455,11 @@
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>2026-02-01~2026-02-28</t>
+          <t>2026-07-01~2026-07-31</t>
         </is>
       </c>
       <c r="D15" t="n">
-        <v>28</v>
+        <v>31</v>
       </c>
       <c r="E15" t="inlineStr">
         <is>
@@ -1519,11 +1519,11 @@
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>2026-02-01~2026-02-28</t>
+          <t>2026-07-01~2026-07-31</t>
         </is>
       </c>
       <c r="D16" t="n">
-        <v>28</v>
+        <v>31</v>
       </c>
       <c r="E16" t="inlineStr">
         <is>
@@ -1583,11 +1583,11 @@
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>2026-02-01~2026-02-28</t>
+          <t>2026-07-01~2026-07-31</t>
         </is>
       </c>
       <c r="D17" t="n">
-        <v>28</v>
+        <v>31</v>
       </c>
       <c r="E17" t="inlineStr">
         <is>
@@ -1647,11 +1647,11 @@
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>2026-02-01~2026-02-28</t>
+          <t>2026-07-01~2026-07-31</t>
         </is>
       </c>
       <c r="D18" t="n">
-        <v>28</v>
+        <v>31</v>
       </c>
       <c r="E18" t="inlineStr">
         <is>
@@ -1711,11 +1711,11 @@
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>2026-02-01~2026-02-28</t>
+          <t>2026-07-01~2026-07-31</t>
         </is>
       </c>
       <c r="D19" t="n">
-        <v>28</v>
+        <v>31</v>
       </c>
       <c r="E19" t="inlineStr">
         <is>
@@ -1775,11 +1775,11 @@
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>2026-02-01~2026-02-28</t>
+          <t>2026-07-01~2026-07-31</t>
         </is>
       </c>
       <c r="D20" t="n">
-        <v>28</v>
+        <v>31</v>
       </c>
       <c r="E20" t="inlineStr">
         <is>
@@ -1829,21 +1829,21 @@
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>ZW01622</t>
+          <t>ZW02547</t>
         </is>
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>Saga Fusion</t>
+          <t>Hong Kong City Restaurant</t>
         </is>
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>2026-02-01~2026-02-28</t>
+          <t>2026-07-01~2026-07-31</t>
         </is>
       </c>
       <c r="D21" t="n">
-        <v>28</v>
+        <v>31</v>
       </c>
       <c r="E21" t="inlineStr">
         <is>
@@ -1856,20 +1856,20 @@
         </is>
       </c>
       <c r="G21" t="n">
-        <v>0</v>
+        <v>873</v>
       </c>
       <c r="H21" t="inlineStr"/>
       <c r="I21" t="n">
         <v>0</v>
       </c>
       <c r="J21" t="n">
-        <v>0</v>
+        <v>873</v>
       </c>
       <c r="K21" t="n">
         <v>1</v>
       </c>
       <c r="L21" t="n">
-        <v>0</v>
+        <v>873</v>
       </c>
       <c r="M21" t="inlineStr"/>
       <c r="N21" t="inlineStr"/>
@@ -1897,27 +1897,27 @@
         <v>2000</v>
       </c>
       <c r="V21" t="n">
-        <v>0</v>
+        <v>873</v>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>ZW01622</t>
+          <t>ZW02547</t>
         </is>
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>Saga Fusion</t>
+          <t>Hong Kong City Restaurant</t>
         </is>
       </c>
       <c r="C22" t="inlineStr">
         <is>
-          <t>2026-02-01~2026-02-28</t>
+          <t>2026-07-01~2026-07-31</t>
         </is>
       </c>
       <c r="D22" t="n">
-        <v>28</v>
+        <v>31</v>
       </c>
       <c r="E22" t="inlineStr">
         <is>
@@ -1930,20 +1930,20 @@
         </is>
       </c>
       <c r="G22" t="n">
-        <v>0</v>
+        <v>377</v>
       </c>
       <c r="H22" t="inlineStr"/>
       <c r="I22" t="n">
         <v>0</v>
       </c>
       <c r="J22" t="n">
-        <v>0</v>
+        <v>377</v>
       </c>
       <c r="K22" t="n">
         <v>1</v>
       </c>
       <c r="L22" t="n">
-        <v>0</v>
+        <v>377</v>
       </c>
       <c r="M22" t="inlineStr"/>
       <c r="N22" t="inlineStr"/>
@@ -1971,27 +1971,27 @@
         <v>1000</v>
       </c>
       <c r="V22" t="n">
-        <v>0</v>
+        <v>377</v>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>ZW01622</t>
+          <t>ZW02547</t>
         </is>
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>Saga Fusion</t>
+          <t>Hong Kong City Restaurant</t>
         </is>
       </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t>2026-02-01~2026-02-28</t>
+          <t>2026-07-01~2026-07-31</t>
         </is>
       </c>
       <c r="D23" t="n">
-        <v>28</v>
+        <v>31</v>
       </c>
       <c r="E23" t="inlineStr">
         <is>
@@ -2004,20 +2004,20 @@
         </is>
       </c>
       <c r="G23" t="n">
-        <v>0</v>
+        <v>463</v>
       </c>
       <c r="H23" t="inlineStr"/>
       <c r="I23" t="n">
         <v>0</v>
       </c>
       <c r="J23" t="n">
-        <v>0</v>
+        <v>463</v>
       </c>
       <c r="K23" t="n">
         <v>1</v>
       </c>
       <c r="L23" t="n">
-        <v>0</v>
+        <v>463</v>
       </c>
       <c r="M23" t="inlineStr"/>
       <c r="N23" t="inlineStr"/>
@@ -2045,27 +2045,27 @@
         <v>500</v>
       </c>
       <c r="V23" t="n">
-        <v>0</v>
+        <v>13.89</v>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>ZW01622</t>
+          <t>ZW02547</t>
         </is>
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>Saga Fusion</t>
+          <t>Hong Kong City Restaurant</t>
         </is>
       </c>
       <c r="C24" t="inlineStr">
         <is>
-          <t>2026-02-01~2026-02-28</t>
+          <t>2026-07-01~2026-07-31</t>
         </is>
       </c>
       <c r="D24" t="n">
-        <v>28</v>
+        <v>31</v>
       </c>
       <c r="E24" t="inlineStr">
         <is>
@@ -2078,20 +2078,20 @@
         </is>
       </c>
       <c r="G24" t="n">
-        <v>0</v>
+        <v>1638</v>
       </c>
       <c r="H24" t="inlineStr"/>
       <c r="I24" t="n">
         <v>0</v>
       </c>
       <c r="J24" t="n">
-        <v>0</v>
+        <v>1638</v>
       </c>
       <c r="K24" t="n">
         <v>1</v>
       </c>
       <c r="L24" t="n">
-        <v>0</v>
+        <v>1638</v>
       </c>
       <c r="M24" t="inlineStr"/>
       <c r="N24" t="inlineStr"/>
@@ -2109,27 +2109,27 @@
       <c r="T24" t="inlineStr"/>
       <c r="U24" t="inlineStr"/>
       <c r="V24" t="n">
-        <v>0</v>
+        <v>1638</v>
       </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>ZW01622</t>
+          <t>ZW02547</t>
         </is>
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>Saga Fusion</t>
+          <t>Hong Kong City Restaurant</t>
         </is>
       </c>
       <c r="C25" t="inlineStr">
         <is>
-          <t>2026-02-01~2026-02-28</t>
+          <t>2026-07-01~2026-07-31</t>
         </is>
       </c>
       <c r="D25" t="n">
-        <v>28</v>
+        <v>31</v>
       </c>
       <c r="E25" t="inlineStr">
         <is>
@@ -2142,20 +2142,20 @@
         </is>
       </c>
       <c r="G25" t="n">
-        <v>0</v>
+        <v>1118</v>
       </c>
       <c r="H25" t="inlineStr"/>
       <c r="I25" t="n">
         <v>0</v>
       </c>
       <c r="J25" t="n">
-        <v>0</v>
+        <v>1118</v>
       </c>
       <c r="K25" t="n">
         <v>1</v>
       </c>
       <c r="L25" t="n">
-        <v>0</v>
+        <v>1118</v>
       </c>
       <c r="M25" t="inlineStr"/>
       <c r="N25" t="inlineStr"/>
@@ -2183,27 +2183,27 @@
         <v>500</v>
       </c>
       <c r="V25" t="n">
-        <v>0</v>
+        <v>33.54</v>
       </c>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>ZW01622</t>
+          <t>ZW02547</t>
         </is>
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>Saga Fusion</t>
+          <t>Hong Kong City Restaurant</t>
         </is>
       </c>
       <c r="C26" t="inlineStr">
         <is>
-          <t>2026-02-01~2026-02-28</t>
+          <t>2026-07-01~2026-07-31</t>
         </is>
       </c>
       <c r="D26" t="n">
-        <v>28</v>
+        <v>31</v>
       </c>
       <c r="E26" t="inlineStr">
         <is>
@@ -2216,20 +2216,20 @@
         </is>
       </c>
       <c r="G26" t="n">
-        <v>0</v>
+        <v>870</v>
       </c>
       <c r="H26" t="inlineStr"/>
       <c r="I26" t="n">
         <v>0</v>
       </c>
       <c r="J26" t="n">
-        <v>0</v>
+        <v>870</v>
       </c>
       <c r="K26" t="n">
         <v>1</v>
       </c>
       <c r="L26" t="n">
-        <v>0</v>
+        <v>870</v>
       </c>
       <c r="M26" t="inlineStr"/>
       <c r="N26" t="inlineStr"/>
@@ -2257,27 +2257,27 @@
         <v>2000</v>
       </c>
       <c r="V26" t="n">
-        <v>0</v>
+        <v>870</v>
       </c>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>ZW01622</t>
+          <t>ZW02547</t>
         </is>
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>Saga Fusion</t>
+          <t>Hong Kong City Restaurant</t>
         </is>
       </c>
       <c r="C27" t="inlineStr">
         <is>
-          <t>2026-02-01~2026-02-28</t>
+          <t>2026-07-01~2026-07-31</t>
         </is>
       </c>
       <c r="D27" t="n">
-        <v>28</v>
+        <v>31</v>
       </c>
       <c r="E27" t="inlineStr">
         <is>
@@ -2290,20 +2290,20 @@
         </is>
       </c>
       <c r="G27" t="n">
-        <v>0</v>
+        <v>145</v>
       </c>
       <c r="H27" t="inlineStr"/>
       <c r="I27" t="n">
         <v>0</v>
       </c>
       <c r="J27" t="n">
-        <v>0</v>
+        <v>145</v>
       </c>
       <c r="K27" t="n">
         <v>1</v>
       </c>
       <c r="L27" t="n">
-        <v>0</v>
+        <v>145</v>
       </c>
       <c r="M27" t="inlineStr"/>
       <c r="N27" t="inlineStr"/>
@@ -2331,27 +2331,27 @@
         <v>2000</v>
       </c>
       <c r="V27" t="n">
-        <v>0</v>
+        <v>145</v>
       </c>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>ZW01622</t>
+          <t>ZW02547</t>
         </is>
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>Saga Fusion</t>
+          <t>Hong Kong City Restaurant</t>
         </is>
       </c>
       <c r="C28" t="inlineStr">
         <is>
-          <t>2026-02-01~2026-02-28</t>
+          <t>2026-07-01~2026-07-31</t>
         </is>
       </c>
       <c r="D28" t="n">
-        <v>28</v>
+        <v>31</v>
       </c>
       <c r="E28" t="inlineStr">
         <is>
@@ -2401,21 +2401,21 @@
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>ZW01622</t>
+          <t>ZW02547</t>
         </is>
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>Saga Fusion</t>
+          <t>Hong Kong City Restaurant</t>
         </is>
       </c>
       <c r="C29" t="inlineStr">
         <is>
-          <t>2026-02-01~2026-02-28</t>
+          <t>2026-07-01~2026-07-31</t>
         </is>
       </c>
       <c r="D29" t="n">
-        <v>28</v>
+        <v>31</v>
       </c>
       <c r="E29" t="inlineStr">
         <is>
@@ -2428,20 +2428,20 @@
         </is>
       </c>
       <c r="G29" t="n">
-        <v>0</v>
+        <v>400</v>
       </c>
       <c r="H29" t="inlineStr"/>
       <c r="I29" t="n">
         <v>0</v>
       </c>
       <c r="J29" t="n">
-        <v>0</v>
+        <v>400</v>
       </c>
       <c r="K29" t="n">
         <v>1</v>
       </c>
       <c r="L29" t="n">
-        <v>0</v>
+        <v>400</v>
       </c>
       <c r="M29" t="inlineStr"/>
       <c r="N29" t="inlineStr"/>
@@ -2469,27 +2469,27 @@
         <v>2000</v>
       </c>
       <c r="V29" t="n">
-        <v>0</v>
+        <v>400</v>
       </c>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>ZW01622</t>
+          <t>ZW02547</t>
         </is>
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t>Saga Fusion</t>
+          <t>Hong Kong City Restaurant</t>
         </is>
       </c>
       <c r="C30" t="inlineStr">
         <is>
-          <t>2026-02-01~2026-02-28</t>
+          <t>2026-07-01~2026-07-31</t>
         </is>
       </c>
       <c r="D30" t="n">
-        <v>28</v>
+        <v>31</v>
       </c>
       <c r="E30" t="inlineStr">
         <is>
@@ -2539,21 +2539,21 @@
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>ZW01622</t>
+          <t>ZW02547</t>
         </is>
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>Saga Fusion</t>
+          <t>Hong Kong City Restaurant</t>
         </is>
       </c>
       <c r="C31" t="inlineStr">
         <is>
-          <t>2026-02-01~2026-02-28</t>
+          <t>2026-07-01~2026-07-31</t>
         </is>
       </c>
       <c r="D31" t="n">
-        <v>28</v>
+        <v>31</v>
       </c>
       <c r="E31" t="inlineStr">
         <is>
@@ -2603,21 +2603,21 @@
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>ZW01622</t>
+          <t>ZW02547</t>
         </is>
       </c>
       <c r="B32" t="inlineStr">
         <is>
-          <t>Saga Fusion</t>
+          <t>Hong Kong City Restaurant</t>
         </is>
       </c>
       <c r="C32" t="inlineStr">
         <is>
-          <t>2026-02-01~2026-02-28</t>
+          <t>2026-07-01~2026-07-31</t>
         </is>
       </c>
       <c r="D32" t="n">
-        <v>28</v>
+        <v>31</v>
       </c>
       <c r="E32" t="inlineStr">
         <is>
@@ -2667,21 +2667,21 @@
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>ZW01622</t>
+          <t>ZW02547</t>
         </is>
       </c>
       <c r="B33" t="inlineStr">
         <is>
-          <t>Saga Fusion</t>
+          <t>Hong Kong City Restaurant</t>
         </is>
       </c>
       <c r="C33" t="inlineStr">
         <is>
-          <t>2026-02-01~2026-02-28</t>
+          <t>2026-07-01~2026-07-31</t>
         </is>
       </c>
       <c r="D33" t="n">
-        <v>28</v>
+        <v>31</v>
       </c>
       <c r="E33" t="inlineStr">
         <is>
@@ -2731,21 +2731,21 @@
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t>ZW01622</t>
+          <t>ZW02547</t>
         </is>
       </c>
       <c r="B34" t="inlineStr">
         <is>
-          <t>Saga Fusion</t>
+          <t>Hong Kong City Restaurant</t>
         </is>
       </c>
       <c r="C34" t="inlineStr">
         <is>
-          <t>2026-02-01~2026-02-28</t>
+          <t>2026-07-01~2026-07-31</t>
         </is>
       </c>
       <c r="D34" t="n">
-        <v>28</v>
+        <v>31</v>
       </c>
       <c r="E34" t="inlineStr">
         <is>
@@ -2795,21 +2795,21 @@
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>ZW01622</t>
+          <t>ZW02547</t>
         </is>
       </c>
       <c r="B35" t="inlineStr">
         <is>
-          <t>Saga Fusion</t>
+          <t>Hong Kong City Restaurant</t>
         </is>
       </c>
       <c r="C35" t="inlineStr">
         <is>
-          <t>2026-02-01~2026-02-28</t>
+          <t>2026-07-01~2026-07-31</t>
         </is>
       </c>
       <c r="D35" t="n">
-        <v>28</v>
+        <v>31</v>
       </c>
       <c r="E35" t="inlineStr">
         <is>
@@ -2859,21 +2859,21 @@
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
-          <t>ZW01622</t>
+          <t>ZW02547</t>
         </is>
       </c>
       <c r="B36" t="inlineStr">
         <is>
-          <t>Saga Fusion</t>
+          <t>Hong Kong City Restaurant</t>
         </is>
       </c>
       <c r="C36" t="inlineStr">
         <is>
-          <t>2026-02-01~2026-02-28</t>
+          <t>2026-07-01~2026-07-31</t>
         </is>
       </c>
       <c r="D36" t="n">
-        <v>28</v>
+        <v>31</v>
       </c>
       <c r="E36" t="inlineStr">
         <is>
@@ -2923,21 +2923,21 @@
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>ZW01622</t>
+          <t>ZW02547</t>
         </is>
       </c>
       <c r="B37" t="inlineStr">
         <is>
-          <t>Saga Fusion</t>
+          <t>Hong Kong City Restaurant</t>
         </is>
       </c>
       <c r="C37" t="inlineStr">
         <is>
-          <t>2026-02-01~2026-02-28</t>
+          <t>2026-07-01~2026-07-31</t>
         </is>
       </c>
       <c r="D37" t="n">
-        <v>28</v>
+        <v>31</v>
       </c>
       <c r="E37" t="inlineStr">
         <is>
@@ -2987,21 +2987,21 @@
     <row r="38">
       <c r="A38" t="inlineStr">
         <is>
-          <t>ZW01622</t>
+          <t>ZW02547</t>
         </is>
       </c>
       <c r="B38" t="inlineStr">
         <is>
-          <t>Saga Fusion</t>
+          <t>Hong Kong City Restaurant</t>
         </is>
       </c>
       <c r="C38" t="inlineStr">
         <is>
-          <t>2026-02-01~2026-02-28</t>
+          <t>2026-07-01~2026-07-31</t>
         </is>
       </c>
       <c r="D38" t="n">
-        <v>28</v>
+        <v>31</v>
       </c>
       <c r="E38" t="inlineStr">
         <is>
@@ -3051,21 +3051,21 @@
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t>ZW01622</t>
+          <t>ZW02547</t>
         </is>
       </c>
       <c r="B39" t="inlineStr">
         <is>
-          <t>Saga Fusion</t>
+          <t>Hong Kong City Restaurant</t>
         </is>
       </c>
       <c r="C39" t="inlineStr">
         <is>
-          <t>2026-02-01~2026-02-28</t>
+          <t>2026-07-01~2026-07-31</t>
         </is>
       </c>
       <c r="D39" t="n">
-        <v>28</v>
+        <v>31</v>
       </c>
       <c r="E39" t="inlineStr">
         <is>
@@ -3115,21 +3115,21 @@
     <row r="40">
       <c r="A40" t="inlineStr">
         <is>
-          <t>ZW01654</t>
+          <t>ZW01622</t>
         </is>
       </c>
       <c r="B40" t="inlineStr">
         <is>
-          <t>Thyme Japanese Cuisine</t>
+          <t>Saga Fusion</t>
         </is>
       </c>
       <c r="C40" t="inlineStr">
         <is>
-          <t>2026-02-01~2026-02-28</t>
+          <t>2026-07-01~2026-07-31</t>
         </is>
       </c>
       <c r="D40" t="n">
-        <v>28</v>
+        <v>31</v>
       </c>
       <c r="E40" t="inlineStr">
         <is>
@@ -3142,20 +3142,20 @@
         </is>
       </c>
       <c r="G40" t="n">
-        <v>2650</v>
+        <v>9569</v>
       </c>
       <c r="H40" t="inlineStr"/>
       <c r="I40" t="n">
         <v>0</v>
       </c>
       <c r="J40" t="n">
-        <v>2650</v>
+        <v>9569</v>
       </c>
       <c r="K40" t="n">
         <v>1</v>
       </c>
       <c r="L40" t="n">
-        <v>2650</v>
+        <v>9569</v>
       </c>
       <c r="M40" t="inlineStr"/>
       <c r="N40" t="inlineStr"/>
@@ -3183,27 +3183,27 @@
         <v>2000</v>
       </c>
       <c r="V40" t="n">
-        <v>2650</v>
+        <v>9569</v>
       </c>
     </row>
     <row r="41">
       <c r="A41" t="inlineStr">
         <is>
-          <t>ZW01654</t>
+          <t>ZW01622</t>
         </is>
       </c>
       <c r="B41" t="inlineStr">
         <is>
-          <t>Thyme Japanese Cuisine</t>
+          <t>Saga Fusion</t>
         </is>
       </c>
       <c r="C41" t="inlineStr">
         <is>
-          <t>2026-02-01~2026-02-28</t>
+          <t>2026-07-01~2026-07-31</t>
         </is>
       </c>
       <c r="D41" t="n">
-        <v>28</v>
+        <v>31</v>
       </c>
       <c r="E41" t="inlineStr">
         <is>
@@ -3216,20 +3216,20 @@
         </is>
       </c>
       <c r="G41" t="n">
-        <v>9245</v>
+        <v>22853</v>
       </c>
       <c r="H41" t="inlineStr"/>
       <c r="I41" t="n">
         <v>0</v>
       </c>
       <c r="J41" t="n">
-        <v>9245</v>
+        <v>22853</v>
       </c>
       <c r="K41" t="n">
         <v>1</v>
       </c>
       <c r="L41" t="n">
-        <v>9245</v>
+        <v>22853</v>
       </c>
       <c r="M41" t="inlineStr"/>
       <c r="N41" t="inlineStr"/>
@@ -3257,27 +3257,27 @@
         <v>1000</v>
       </c>
       <c r="V41" t="n">
-        <v>9245</v>
+        <v>22853</v>
       </c>
     </row>
     <row r="42">
       <c r="A42" t="inlineStr">
         <is>
-          <t>ZW01654</t>
+          <t>ZW01622</t>
         </is>
       </c>
       <c r="B42" t="inlineStr">
         <is>
-          <t>Thyme Japanese Cuisine</t>
+          <t>Saga Fusion</t>
         </is>
       </c>
       <c r="C42" t="inlineStr">
         <is>
-          <t>2026-02-01~2026-02-28</t>
+          <t>2026-07-01~2026-07-31</t>
         </is>
       </c>
       <c r="D42" t="n">
-        <v>28</v>
+        <v>31</v>
       </c>
       <c r="E42" t="inlineStr">
         <is>
@@ -3290,20 +3290,20 @@
         </is>
       </c>
       <c r="G42" t="n">
-        <v>24535</v>
+        <v>50229</v>
       </c>
       <c r="H42" t="inlineStr"/>
       <c r="I42" t="n">
         <v>0</v>
       </c>
       <c r="J42" t="n">
-        <v>24535</v>
+        <v>50229</v>
       </c>
       <c r="K42" t="n">
         <v>1</v>
       </c>
       <c r="L42" t="n">
-        <v>24535</v>
+        <v>50229</v>
       </c>
       <c r="M42" t="inlineStr"/>
       <c r="N42" t="inlineStr"/>
@@ -3331,27 +3331,27 @@
         <v>500</v>
       </c>
       <c r="V42" t="n">
-        <v>736.05</v>
+        <v>1506.87</v>
       </c>
     </row>
     <row r="43">
       <c r="A43" t="inlineStr">
         <is>
-          <t>ZW01654</t>
+          <t>ZW01622</t>
         </is>
       </c>
       <c r="B43" t="inlineStr">
         <is>
-          <t>Thyme Japanese Cuisine</t>
+          <t>Saga Fusion</t>
         </is>
       </c>
       <c r="C43" t="inlineStr">
         <is>
-          <t>2026-02-01~2026-02-28</t>
+          <t>2026-07-01~2026-07-31</t>
         </is>
       </c>
       <c r="D43" t="n">
-        <v>28</v>
+        <v>31</v>
       </c>
       <c r="E43" t="inlineStr">
         <is>
@@ -3364,20 +3364,20 @@
         </is>
       </c>
       <c r="G43" t="n">
-        <v>30105</v>
+        <v>95849</v>
       </c>
       <c r="H43" t="inlineStr"/>
       <c r="I43" t="n">
         <v>0</v>
       </c>
       <c r="J43" t="n">
-        <v>30105</v>
+        <v>95849</v>
       </c>
       <c r="K43" t="n">
         <v>1</v>
       </c>
       <c r="L43" t="n">
-        <v>30105</v>
+        <v>95849</v>
       </c>
       <c r="M43" t="inlineStr"/>
       <c r="N43" t="inlineStr"/>
@@ -3395,27 +3395,27 @@
       <c r="T43" t="inlineStr"/>
       <c r="U43" t="inlineStr"/>
       <c r="V43" t="n">
-        <v>30105</v>
+        <v>95849</v>
       </c>
     </row>
     <row r="44">
       <c r="A44" t="inlineStr">
         <is>
-          <t>ZW01654</t>
+          <t>ZW01622</t>
         </is>
       </c>
       <c r="B44" t="inlineStr">
         <is>
-          <t>Thyme Japanese Cuisine</t>
+          <t>Saga Fusion</t>
         </is>
       </c>
       <c r="C44" t="inlineStr">
         <is>
-          <t>2026-02-01~2026-02-28</t>
+          <t>2026-07-01~2026-07-31</t>
         </is>
       </c>
       <c r="D44" t="n">
-        <v>28</v>
+        <v>31</v>
       </c>
       <c r="E44" t="inlineStr">
         <is>
@@ -3428,20 +3428,20 @@
         </is>
       </c>
       <c r="G44" t="n">
-        <v>18540</v>
+        <v>73351</v>
       </c>
       <c r="H44" t="inlineStr"/>
       <c r="I44" t="n">
         <v>0</v>
       </c>
       <c r="J44" t="n">
-        <v>18540</v>
+        <v>73351</v>
       </c>
       <c r="K44" t="n">
         <v>1</v>
       </c>
       <c r="L44" t="n">
-        <v>18540</v>
+        <v>73351</v>
       </c>
       <c r="M44" t="inlineStr"/>
       <c r="N44" t="inlineStr"/>
@@ -3469,27 +3469,27 @@
         <v>500</v>
       </c>
       <c r="V44" t="n">
-        <v>556.2</v>
+        <v>2200.53</v>
       </c>
     </row>
     <row r="45">
       <c r="A45" t="inlineStr">
         <is>
-          <t>ZW01654</t>
+          <t>ZW01622</t>
         </is>
       </c>
       <c r="B45" t="inlineStr">
         <is>
-          <t>Thyme Japanese Cuisine</t>
+          <t>Saga Fusion</t>
         </is>
       </c>
       <c r="C45" t="inlineStr">
         <is>
-          <t>2026-02-01~2026-02-28</t>
+          <t>2026-07-01~2026-07-31</t>
         </is>
       </c>
       <c r="D45" t="n">
-        <v>28</v>
+        <v>31</v>
       </c>
       <c r="E45" t="inlineStr">
         <is>
@@ -3502,20 +3502,20 @@
         </is>
       </c>
       <c r="G45" t="n">
-        <v>4792</v>
+        <v>8810</v>
       </c>
       <c r="H45" t="inlineStr"/>
       <c r="I45" t="n">
         <v>0</v>
       </c>
       <c r="J45" t="n">
-        <v>4792</v>
+        <v>8810</v>
       </c>
       <c r="K45" t="n">
         <v>1</v>
       </c>
       <c r="L45" t="n">
-        <v>4792</v>
+        <v>8810</v>
       </c>
       <c r="M45" t="inlineStr"/>
       <c r="N45" t="inlineStr"/>
@@ -3543,27 +3543,27 @@
         <v>2000</v>
       </c>
       <c r="V45" t="n">
-        <v>4792</v>
+        <v>8810</v>
       </c>
     </row>
     <row r="46">
       <c r="A46" t="inlineStr">
         <is>
-          <t>ZW01654</t>
+          <t>ZW01622</t>
         </is>
       </c>
       <c r="B46" t="inlineStr">
         <is>
-          <t>Thyme Japanese Cuisine</t>
+          <t>Saga Fusion</t>
         </is>
       </c>
       <c r="C46" t="inlineStr">
         <is>
-          <t>2026-02-01~2026-02-28</t>
+          <t>2026-07-01~2026-07-31</t>
         </is>
       </c>
       <c r="D46" t="n">
-        <v>28</v>
+        <v>31</v>
       </c>
       <c r="E46" t="inlineStr">
         <is>
@@ -3576,20 +3576,20 @@
         </is>
       </c>
       <c r="G46" t="n">
-        <v>3945</v>
+        <v>5680</v>
       </c>
       <c r="H46" t="inlineStr"/>
       <c r="I46" t="n">
         <v>0</v>
       </c>
       <c r="J46" t="n">
-        <v>3945</v>
+        <v>5680</v>
       </c>
       <c r="K46" t="n">
         <v>1</v>
       </c>
       <c r="L46" t="n">
-        <v>3945</v>
+        <v>5680</v>
       </c>
       <c r="M46" t="inlineStr"/>
       <c r="N46" t="inlineStr"/>
@@ -3617,27 +3617,27 @@
         <v>2000</v>
       </c>
       <c r="V46" t="n">
-        <v>3945</v>
+        <v>5680</v>
       </c>
     </row>
     <row r="47">
       <c r="A47" t="inlineStr">
         <is>
-          <t>ZW01654</t>
+          <t>ZW01622</t>
         </is>
       </c>
       <c r="B47" t="inlineStr">
         <is>
-          <t>Thyme Japanese Cuisine</t>
+          <t>Saga Fusion</t>
         </is>
       </c>
       <c r="C47" t="inlineStr">
         <is>
-          <t>2026-02-01~2026-02-28</t>
+          <t>2026-07-01~2026-07-31</t>
         </is>
       </c>
       <c r="D47" t="n">
-        <v>28</v>
+        <v>31</v>
       </c>
       <c r="E47" t="inlineStr">
         <is>
@@ -3650,20 +3650,20 @@
         </is>
       </c>
       <c r="G47" t="n">
-        <v>0</v>
+        <v>5115</v>
       </c>
       <c r="H47" t="inlineStr"/>
       <c r="I47" t="n">
         <v>0</v>
       </c>
       <c r="J47" t="n">
-        <v>0</v>
+        <v>5115</v>
       </c>
       <c r="K47" t="n">
         <v>1</v>
       </c>
       <c r="L47" t="n">
-        <v>0</v>
+        <v>5115</v>
       </c>
       <c r="M47" t="inlineStr"/>
       <c r="N47" t="inlineStr"/>
@@ -3681,27 +3681,27 @@
       <c r="T47" t="inlineStr"/>
       <c r="U47" t="inlineStr"/>
       <c r="V47" t="n">
-        <v>0</v>
+        <v>5115</v>
       </c>
     </row>
     <row r="48">
       <c r="A48" t="inlineStr">
         <is>
-          <t>ZW01654</t>
+          <t>ZW01622</t>
         </is>
       </c>
       <c r="B48" t="inlineStr">
         <is>
-          <t>Thyme Japanese Cuisine</t>
+          <t>Saga Fusion</t>
         </is>
       </c>
       <c r="C48" t="inlineStr">
         <is>
-          <t>2026-02-01~2026-02-28</t>
+          <t>2026-07-01~2026-07-31</t>
         </is>
       </c>
       <c r="D48" t="n">
-        <v>28</v>
+        <v>31</v>
       </c>
       <c r="E48" t="inlineStr">
         <is>
@@ -3714,20 +3714,20 @@
         </is>
       </c>
       <c r="G48" t="n">
-        <v>7500</v>
+        <v>7667</v>
       </c>
       <c r="H48" t="inlineStr"/>
       <c r="I48" t="n">
         <v>0</v>
       </c>
       <c r="J48" t="n">
-        <v>7500</v>
+        <v>7667</v>
       </c>
       <c r="K48" t="n">
         <v>1</v>
       </c>
       <c r="L48" t="n">
-        <v>7500</v>
+        <v>7667</v>
       </c>
       <c r="M48" t="inlineStr"/>
       <c r="N48" t="inlineStr"/>
@@ -3755,27 +3755,27 @@
         <v>2000</v>
       </c>
       <c r="V48" t="n">
-        <v>7500</v>
+        <v>7667</v>
       </c>
     </row>
     <row r="49">
       <c r="A49" t="inlineStr">
         <is>
-          <t>ZW01654</t>
+          <t>ZW01622</t>
         </is>
       </c>
       <c r="B49" t="inlineStr">
         <is>
-          <t>Thyme Japanese Cuisine</t>
+          <t>Saga Fusion</t>
         </is>
       </c>
       <c r="C49" t="inlineStr">
         <is>
-          <t>2026-02-01~2026-02-28</t>
+          <t>2026-07-01~2026-07-31</t>
         </is>
       </c>
       <c r="D49" t="n">
-        <v>28</v>
+        <v>31</v>
       </c>
       <c r="E49" t="inlineStr">
         <is>
@@ -3788,20 +3788,20 @@
         </is>
       </c>
       <c r="G49" t="n">
-        <v>3055</v>
+        <v>0</v>
       </c>
       <c r="H49" t="inlineStr"/>
       <c r="I49" t="n">
         <v>0</v>
       </c>
       <c r="J49" t="n">
-        <v>3055</v>
+        <v>0</v>
       </c>
       <c r="K49" t="n">
         <v>1</v>
       </c>
       <c r="L49" t="n">
-        <v>3055</v>
+        <v>0</v>
       </c>
       <c r="M49" t="inlineStr"/>
       <c r="N49" t="inlineStr"/>
@@ -3819,27 +3819,27 @@
       <c r="T49" t="inlineStr"/>
       <c r="U49" t="inlineStr"/>
       <c r="V49" t="n">
-        <v>3055</v>
+        <v>0</v>
       </c>
     </row>
     <row r="50">
       <c r="A50" t="inlineStr">
         <is>
-          <t>ZW01654</t>
+          <t>ZW01622</t>
         </is>
       </c>
       <c r="B50" t="inlineStr">
         <is>
-          <t>Thyme Japanese Cuisine</t>
+          <t>Saga Fusion</t>
         </is>
       </c>
       <c r="C50" t="inlineStr">
         <is>
-          <t>2026-02-01~2026-02-28</t>
+          <t>2026-07-01~2026-07-31</t>
         </is>
       </c>
       <c r="D50" t="n">
-        <v>28</v>
+        <v>31</v>
       </c>
       <c r="E50" t="inlineStr">
         <is>
@@ -3889,21 +3889,21 @@
     <row r="51">
       <c r="A51" t="inlineStr">
         <is>
-          <t>ZW01654</t>
+          <t>ZW01622</t>
         </is>
       </c>
       <c r="B51" t="inlineStr">
         <is>
-          <t>Thyme Japanese Cuisine</t>
+          <t>Saga Fusion</t>
         </is>
       </c>
       <c r="C51" t="inlineStr">
         <is>
-          <t>2026-02-01~2026-02-28</t>
+          <t>2026-07-01~2026-07-31</t>
         </is>
       </c>
       <c r="D51" t="n">
-        <v>28</v>
+        <v>31</v>
       </c>
       <c r="E51" t="inlineStr">
         <is>
@@ -3953,21 +3953,21 @@
     <row r="52">
       <c r="A52" t="inlineStr">
         <is>
-          <t>ZW01654</t>
+          <t>ZW01622</t>
         </is>
       </c>
       <c r="B52" t="inlineStr">
         <is>
-          <t>Thyme Japanese Cuisine</t>
+          <t>Saga Fusion</t>
         </is>
       </c>
       <c r="C52" t="inlineStr">
         <is>
-          <t>2026-02-01~2026-02-28</t>
+          <t>2026-07-01~2026-07-31</t>
         </is>
       </c>
       <c r="D52" t="n">
-        <v>28</v>
+        <v>31</v>
       </c>
       <c r="E52" t="inlineStr">
         <is>
@@ -4017,21 +4017,21 @@
     <row r="53">
       <c r="A53" t="inlineStr">
         <is>
-          <t>ZW01654</t>
+          <t>ZW01622</t>
         </is>
       </c>
       <c r="B53" t="inlineStr">
         <is>
-          <t>Thyme Japanese Cuisine</t>
+          <t>Saga Fusion</t>
         </is>
       </c>
       <c r="C53" t="inlineStr">
         <is>
-          <t>2026-02-01~2026-02-28</t>
+          <t>2026-07-01~2026-07-31</t>
         </is>
       </c>
       <c r="D53" t="n">
-        <v>28</v>
+        <v>31</v>
       </c>
       <c r="E53" t="inlineStr">
         <is>
@@ -4044,20 +4044,20 @@
         </is>
       </c>
       <c r="G53" t="n">
-        <v>0</v>
+        <v>10082</v>
       </c>
       <c r="H53" t="inlineStr"/>
       <c r="I53" t="n">
         <v>0</v>
       </c>
       <c r="J53" t="n">
-        <v>0</v>
+        <v>10082</v>
       </c>
       <c r="K53" t="n">
         <v>1</v>
       </c>
       <c r="L53" t="n">
-        <v>0</v>
+        <v>10082</v>
       </c>
       <c r="M53" t="inlineStr"/>
       <c r="N53" t="inlineStr"/>
@@ -4075,27 +4075,27 @@
       <c r="T53" t="inlineStr"/>
       <c r="U53" t="inlineStr"/>
       <c r="V53" t="n">
-        <v>0</v>
+        <v>10082</v>
       </c>
     </row>
     <row r="54">
       <c r="A54" t="inlineStr">
         <is>
-          <t>ZW01654</t>
+          <t>ZW01622</t>
         </is>
       </c>
       <c r="B54" t="inlineStr">
         <is>
-          <t>Thyme Japanese Cuisine</t>
+          <t>Saga Fusion</t>
         </is>
       </c>
       <c r="C54" t="inlineStr">
         <is>
-          <t>2026-02-01~2026-02-28</t>
+          <t>2026-07-01~2026-07-31</t>
         </is>
       </c>
       <c r="D54" t="n">
-        <v>28</v>
+        <v>31</v>
       </c>
       <c r="E54" t="inlineStr">
         <is>
@@ -4145,21 +4145,21 @@
     <row r="55">
       <c r="A55" t="inlineStr">
         <is>
-          <t>ZW01654</t>
+          <t>ZW01622</t>
         </is>
       </c>
       <c r="B55" t="inlineStr">
         <is>
-          <t>Thyme Japanese Cuisine</t>
+          <t>Saga Fusion</t>
         </is>
       </c>
       <c r="C55" t="inlineStr">
         <is>
-          <t>2026-02-01~2026-02-28</t>
+          <t>2026-07-01~2026-07-31</t>
         </is>
       </c>
       <c r="D55" t="n">
-        <v>28</v>
+        <v>31</v>
       </c>
       <c r="E55" t="inlineStr">
         <is>
@@ -4209,21 +4209,21 @@
     <row r="56">
       <c r="A56" t="inlineStr">
         <is>
-          <t>ZW01654</t>
+          <t>ZW01622</t>
         </is>
       </c>
       <c r="B56" t="inlineStr">
         <is>
-          <t>Thyme Japanese Cuisine</t>
+          <t>Saga Fusion</t>
         </is>
       </c>
       <c r="C56" t="inlineStr">
         <is>
-          <t>2026-02-01~2026-02-28</t>
+          <t>2026-07-01~2026-07-31</t>
         </is>
       </c>
       <c r="D56" t="n">
-        <v>28</v>
+        <v>31</v>
       </c>
       <c r="E56" t="inlineStr">
         <is>
@@ -4273,21 +4273,21 @@
     <row r="57">
       <c r="A57" t="inlineStr">
         <is>
-          <t>ZW01654</t>
+          <t>ZW01622</t>
         </is>
       </c>
       <c r="B57" t="inlineStr">
         <is>
-          <t>Thyme Japanese Cuisine</t>
+          <t>Saga Fusion</t>
         </is>
       </c>
       <c r="C57" t="inlineStr">
         <is>
-          <t>2026-02-01~2026-02-28</t>
+          <t>2026-07-01~2026-07-31</t>
         </is>
       </c>
       <c r="D57" t="n">
-        <v>28</v>
+        <v>31</v>
       </c>
       <c r="E57" t="inlineStr">
         <is>
@@ -4337,21 +4337,21 @@
     <row r="58">
       <c r="A58" t="inlineStr">
         <is>
-          <t>ZW01654</t>
+          <t>ZW01622</t>
         </is>
       </c>
       <c r="B58" t="inlineStr">
         <is>
-          <t>Thyme Japanese Cuisine</t>
+          <t>Saga Fusion</t>
         </is>
       </c>
       <c r="C58" t="inlineStr">
         <is>
-          <t>2026-02-01~2026-02-28</t>
+          <t>2026-07-01~2026-07-31</t>
         </is>
       </c>
       <c r="D58" t="n">
-        <v>28</v>
+        <v>31</v>
       </c>
       <c r="E58" t="inlineStr">
         <is>
@@ -4364,20 +4364,20 @@
         </is>
       </c>
       <c r="G58" t="n">
-        <v>0</v>
+        <v>2545</v>
       </c>
       <c r="H58" t="inlineStr"/>
       <c r="I58" t="n">
         <v>0</v>
       </c>
       <c r="J58" t="n">
-        <v>0</v>
+        <v>2545</v>
       </c>
       <c r="K58" t="n">
         <v>1</v>
       </c>
       <c r="L58" t="n">
-        <v>0</v>
+        <v>2545</v>
       </c>
       <c r="M58" t="inlineStr"/>
       <c r="N58" t="inlineStr"/>
@@ -4395,6 +4395,2578 @@
       <c r="T58" t="inlineStr"/>
       <c r="U58" t="inlineStr"/>
       <c r="V58" t="n">
+        <v>2545</v>
+      </c>
+    </row>
+    <row r="59">
+      <c r="A59" t="inlineStr">
+        <is>
+          <t>ZW01654</t>
+        </is>
+      </c>
+      <c r="B59" t="inlineStr">
+        <is>
+          <t>Thyme Japanese Cuisine</t>
+        </is>
+      </c>
+      <c r="C59" t="inlineStr">
+        <is>
+          <t>2026-07-01~2026-07-31</t>
+        </is>
+      </c>
+      <c r="D59" t="n">
+        <v>31</v>
+      </c>
+      <c r="E59" t="inlineStr">
+        <is>
+          <t>冰糖糖浆 Fructose Syrup</t>
+        </is>
+      </c>
+      <c r="F59" t="inlineStr">
+        <is>
+          <t>M13</t>
+        </is>
+      </c>
+      <c r="G59" t="n">
+        <v>3138</v>
+      </c>
+      <c r="H59" t="inlineStr"/>
+      <c r="I59" t="n">
+        <v>0</v>
+      </c>
+      <c r="J59" t="n">
+        <v>3138</v>
+      </c>
+      <c r="K59" t="n">
+        <v>1</v>
+      </c>
+      <c r="L59" t="n">
+        <v>3138</v>
+      </c>
+      <c r="M59" t="inlineStr"/>
+      <c r="N59" t="inlineStr"/>
+      <c r="O59" t="n">
+        <v>0</v>
+      </c>
+      <c r="P59" t="inlineStr"/>
+      <c r="Q59" t="inlineStr"/>
+      <c r="R59" t="inlineStr">
+        <is>
+          <t>Fructose Syrup</t>
+        </is>
+      </c>
+      <c r="S59" t="inlineStr">
+        <is>
+          <t>18 months</t>
+        </is>
+      </c>
+      <c r="T59" t="inlineStr">
+        <is>
+          <t>$15.60</t>
+        </is>
+      </c>
+      <c r="U59" t="n">
+        <v>2000</v>
+      </c>
+      <c r="V59" t="n">
+        <v>3138</v>
+      </c>
+    </row>
+    <row r="60">
+      <c r="A60" t="inlineStr">
+        <is>
+          <t>ZW01654</t>
+        </is>
+      </c>
+      <c r="B60" t="inlineStr">
+        <is>
+          <t>Thyme Japanese Cuisine</t>
+        </is>
+      </c>
+      <c r="C60" t="inlineStr">
+        <is>
+          <t>2026-07-01~2026-07-31</t>
+        </is>
+      </c>
+      <c r="D60" t="n">
+        <v>31</v>
+      </c>
+      <c r="E60" t="inlineStr">
+        <is>
+          <t>冰勃朗 Ice Blanc</t>
+        </is>
+      </c>
+      <c r="F60" t="inlineStr">
+        <is>
+          <t>M14</t>
+        </is>
+      </c>
+      <c r="G60" t="n">
+        <v>13945</v>
+      </c>
+      <c r="H60" t="inlineStr"/>
+      <c r="I60" t="n">
+        <v>0</v>
+      </c>
+      <c r="J60" t="n">
+        <v>13945</v>
+      </c>
+      <c r="K60" t="n">
+        <v>1</v>
+      </c>
+      <c r="L60" t="n">
+        <v>13945</v>
+      </c>
+      <c r="M60" t="inlineStr"/>
+      <c r="N60" t="inlineStr"/>
+      <c r="O60" t="n">
+        <v>0</v>
+      </c>
+      <c r="P60" t="inlineStr"/>
+      <c r="Q60" t="inlineStr"/>
+      <c r="R60" t="inlineStr">
+        <is>
+          <t>Ice Blanc</t>
+        </is>
+      </c>
+      <c r="S60" t="inlineStr">
+        <is>
+          <t>9 months</t>
+        </is>
+      </c>
+      <c r="T60" t="inlineStr">
+        <is>
+          <t>$12.00</t>
+        </is>
+      </c>
+      <c r="U60" t="n">
+        <v>1000</v>
+      </c>
+      <c r="V60" t="n">
+        <v>13945</v>
+      </c>
+    </row>
+    <row r="61">
+      <c r="A61" t="inlineStr">
+        <is>
+          <t>ZW01654</t>
+        </is>
+      </c>
+      <c r="B61" t="inlineStr">
+        <is>
+          <t>Thyme Japanese Cuisine</t>
+        </is>
+      </c>
+      <c r="C61" t="inlineStr">
+        <is>
+          <t>2026-07-01~2026-07-31</t>
+        </is>
+      </c>
+      <c r="D61" t="n">
+        <v>31</v>
+      </c>
+      <c r="E61" t="inlineStr">
+        <is>
+          <t>锡兰红茶茶汤 Black Tea</t>
+        </is>
+      </c>
+      <c r="F61" t="inlineStr">
+        <is>
+          <t>M16</t>
+        </is>
+      </c>
+      <c r="G61" t="n">
+        <v>35650</v>
+      </c>
+      <c r="H61" t="inlineStr"/>
+      <c r="I61" t="n">
+        <v>0</v>
+      </c>
+      <c r="J61" t="n">
+        <v>35650</v>
+      </c>
+      <c r="K61" t="n">
+        <v>1</v>
+      </c>
+      <c r="L61" t="n">
+        <v>35650</v>
+      </c>
+      <c r="M61" t="inlineStr"/>
+      <c r="N61" t="inlineStr"/>
+      <c r="O61" t="n">
+        <v>0</v>
+      </c>
+      <c r="P61" t="inlineStr"/>
+      <c r="Q61" t="inlineStr"/>
+      <c r="R61" t="inlineStr">
+        <is>
+          <t>Black Tea</t>
+        </is>
+      </c>
+      <c r="S61" t="inlineStr">
+        <is>
+          <t>24 months</t>
+        </is>
+      </c>
+      <c r="T61" t="inlineStr">
+        <is>
+          <t>$12.30</t>
+        </is>
+      </c>
+      <c r="U61" t="n">
+        <v>500</v>
+      </c>
+      <c r="V61" t="n">
+        <v>1069.5</v>
+      </c>
+    </row>
+    <row r="62">
+      <c r="A62" t="inlineStr">
+        <is>
+          <t>ZW01654</t>
+        </is>
+      </c>
+      <c r="B62" t="inlineStr">
+        <is>
+          <t>Thyme Japanese Cuisine</t>
+        </is>
+      </c>
+      <c r="C62" t="inlineStr">
+        <is>
+          <t>2026-07-01~2026-07-31</t>
+        </is>
+      </c>
+      <c r="D62" t="n">
+        <v>31</v>
+      </c>
+      <c r="E62" t="inlineStr">
+        <is>
+          <t>冰水 Cold Water</t>
+        </is>
+      </c>
+      <c r="F62" t="inlineStr">
+        <is>
+          <t>M22</t>
+        </is>
+      </c>
+      <c r="G62" t="n">
+        <v>36101</v>
+      </c>
+      <c r="H62" t="inlineStr"/>
+      <c r="I62" t="n">
+        <v>0</v>
+      </c>
+      <c r="J62" t="n">
+        <v>36101</v>
+      </c>
+      <c r="K62" t="n">
+        <v>1</v>
+      </c>
+      <c r="L62" t="n">
+        <v>36101</v>
+      </c>
+      <c r="M62" t="inlineStr"/>
+      <c r="N62" t="inlineStr"/>
+      <c r="O62" t="n">
+        <v>0</v>
+      </c>
+      <c r="P62" t="inlineStr"/>
+      <c r="Q62" t="inlineStr"/>
+      <c r="R62" t="inlineStr">
+        <is>
+          <t>Cold Water</t>
+        </is>
+      </c>
+      <c r="S62" t="inlineStr"/>
+      <c r="T62" t="inlineStr"/>
+      <c r="U62" t="inlineStr"/>
+      <c r="V62" t="n">
+        <v>36101</v>
+      </c>
+    </row>
+    <row r="63">
+      <c r="A63" t="inlineStr">
+        <is>
+          <t>ZW01654</t>
+        </is>
+      </c>
+      <c r="B63" t="inlineStr">
+        <is>
+          <t>Thyme Japanese Cuisine</t>
+        </is>
+      </c>
+      <c r="C63" t="inlineStr">
+        <is>
+          <t>2026-07-01~2026-07-31</t>
+        </is>
+      </c>
+      <c r="D63" t="n">
+        <v>31</v>
+      </c>
+      <c r="E63" t="inlineStr">
+        <is>
+          <t>茉莉雪芽茶汤 Green Tea</t>
+        </is>
+      </c>
+      <c r="F63" t="inlineStr">
+        <is>
+          <t>M23</t>
+        </is>
+      </c>
+      <c r="G63" t="n">
+        <v>19268</v>
+      </c>
+      <c r="H63" t="inlineStr"/>
+      <c r="I63" t="n">
+        <v>0</v>
+      </c>
+      <c r="J63" t="n">
+        <v>19268</v>
+      </c>
+      <c r="K63" t="n">
+        <v>1</v>
+      </c>
+      <c r="L63" t="n">
+        <v>19268</v>
+      </c>
+      <c r="M63" t="inlineStr"/>
+      <c r="N63" t="inlineStr"/>
+      <c r="O63" t="n">
+        <v>0</v>
+      </c>
+      <c r="P63" t="inlineStr"/>
+      <c r="Q63" t="inlineStr"/>
+      <c r="R63" t="inlineStr">
+        <is>
+          <t>Green Tea</t>
+        </is>
+      </c>
+      <c r="S63" t="inlineStr">
+        <is>
+          <t>24 months</t>
+        </is>
+      </c>
+      <c r="T63" t="inlineStr">
+        <is>
+          <t>$16.20</t>
+        </is>
+      </c>
+      <c r="U63" t="n">
+        <v>500</v>
+      </c>
+      <c r="V63" t="n">
+        <v>578.04</v>
+      </c>
+    </row>
+    <row r="64">
+      <c r="A64" t="inlineStr">
+        <is>
+          <t>ZW01654</t>
+        </is>
+      </c>
+      <c r="B64" t="inlineStr">
+        <is>
+          <t>Thyme Japanese Cuisine</t>
+        </is>
+      </c>
+      <c r="C64" t="inlineStr">
+        <is>
+          <t>2026-07-01~2026-07-31</t>
+        </is>
+      </c>
+      <c r="D64" t="n">
+        <v>31</v>
+      </c>
+      <c r="E64" t="inlineStr">
+        <is>
+          <t>黑糖糖浆 Brown Sugar</t>
+        </is>
+      </c>
+      <c r="F64" t="inlineStr">
+        <is>
+          <t>M27</t>
+        </is>
+      </c>
+      <c r="G64" t="n">
+        <v>5570</v>
+      </c>
+      <c r="H64" t="inlineStr"/>
+      <c r="I64" t="n">
+        <v>0</v>
+      </c>
+      <c r="J64" t="n">
+        <v>5570</v>
+      </c>
+      <c r="K64" t="n">
+        <v>1</v>
+      </c>
+      <c r="L64" t="n">
+        <v>5570</v>
+      </c>
+      <c r="M64" t="inlineStr"/>
+      <c r="N64" t="inlineStr"/>
+      <c r="O64" t="n">
+        <v>0</v>
+      </c>
+      <c r="P64" t="inlineStr"/>
+      <c r="Q64" t="inlineStr"/>
+      <c r="R64" t="inlineStr">
+        <is>
+          <t>Brown Sugar</t>
+        </is>
+      </c>
+      <c r="S64" t="inlineStr">
+        <is>
+          <t>18 months</t>
+        </is>
+      </c>
+      <c r="T64" t="inlineStr">
+        <is>
+          <t>$15.60</t>
+        </is>
+      </c>
+      <c r="U64" t="n">
+        <v>2000</v>
+      </c>
+      <c r="V64" t="n">
+        <v>5570</v>
+      </c>
+    </row>
+    <row r="65">
+      <c r="A65" t="inlineStr">
+        <is>
+          <t>ZW01654</t>
+        </is>
+      </c>
+      <c r="B65" t="inlineStr">
+        <is>
+          <t>Thyme Japanese Cuisine</t>
+        </is>
+      </c>
+      <c r="C65" t="inlineStr">
+        <is>
+          <t>2026-07-01~2026-07-31</t>
+        </is>
+      </c>
+      <c r="D65" t="n">
+        <v>31</v>
+      </c>
+      <c r="E65" t="inlineStr">
+        <is>
+          <t>蜜桃糖浆 Peach Syrup</t>
+        </is>
+      </c>
+      <c r="F65" t="inlineStr">
+        <is>
+          <t>M28</t>
+        </is>
+      </c>
+      <c r="G65" t="n">
+        <v>5300</v>
+      </c>
+      <c r="H65" t="inlineStr"/>
+      <c r="I65" t="n">
+        <v>0</v>
+      </c>
+      <c r="J65" t="n">
+        <v>5300</v>
+      </c>
+      <c r="K65" t="n">
+        <v>1</v>
+      </c>
+      <c r="L65" t="n">
+        <v>5300</v>
+      </c>
+      <c r="M65" t="inlineStr"/>
+      <c r="N65" t="inlineStr"/>
+      <c r="O65" t="n">
+        <v>0</v>
+      </c>
+      <c r="P65" t="inlineStr"/>
+      <c r="Q65" t="inlineStr"/>
+      <c r="R65" t="inlineStr">
+        <is>
+          <t>Peach Syrup</t>
+        </is>
+      </c>
+      <c r="S65" t="inlineStr">
+        <is>
+          <t>18 months</t>
+        </is>
+      </c>
+      <c r="T65" t="inlineStr">
+        <is>
+          <t>$16.80</t>
+        </is>
+      </c>
+      <c r="U65" t="n">
+        <v>2000</v>
+      </c>
+      <c r="V65" t="n">
+        <v>5300</v>
+      </c>
+    </row>
+    <row r="66">
+      <c r="A66" t="inlineStr">
+        <is>
+          <t>ZW01654</t>
+        </is>
+      </c>
+      <c r="B66" t="inlineStr">
+        <is>
+          <t>Thyme Japanese Cuisine</t>
+        </is>
+      </c>
+      <c r="C66" t="inlineStr">
+        <is>
+          <t>2026-07-01~2026-07-31</t>
+        </is>
+      </c>
+      <c r="D66" t="n">
+        <v>31</v>
+      </c>
+      <c r="E66" t="inlineStr">
+        <is>
+          <t>荔枝糖浆 Lychee Syrup</t>
+        </is>
+      </c>
+      <c r="F66" t="inlineStr">
+        <is>
+          <t>M29</t>
+        </is>
+      </c>
+      <c r="G66" t="n">
+        <v>0</v>
+      </c>
+      <c r="H66" t="inlineStr"/>
+      <c r="I66" t="n">
+        <v>0</v>
+      </c>
+      <c r="J66" t="n">
+        <v>0</v>
+      </c>
+      <c r="K66" t="n">
+        <v>1</v>
+      </c>
+      <c r="L66" t="n">
+        <v>0</v>
+      </c>
+      <c r="M66" t="inlineStr"/>
+      <c r="N66" t="inlineStr"/>
+      <c r="O66" t="n">
+        <v>0</v>
+      </c>
+      <c r="P66" t="inlineStr"/>
+      <c r="Q66" t="inlineStr"/>
+      <c r="R66" t="inlineStr">
+        <is>
+          <t>Lychee Syrup</t>
+        </is>
+      </c>
+      <c r="S66" t="inlineStr"/>
+      <c r="T66" t="inlineStr"/>
+      <c r="U66" t="inlineStr"/>
+      <c r="V66" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="67">
+      <c r="A67" t="inlineStr">
+        <is>
+          <t>ZW01654</t>
+        </is>
+      </c>
+      <c r="B67" t="inlineStr">
+        <is>
+          <t>Thyme Japanese Cuisine</t>
+        </is>
+      </c>
+      <c r="C67" t="inlineStr">
+        <is>
+          <t>2026-07-01~2026-07-31</t>
+        </is>
+      </c>
+      <c r="D67" t="n">
+        <v>31</v>
+      </c>
+      <c r="E67" t="inlineStr">
+        <is>
+          <t>芒果糖浆 Mango Syrup</t>
+        </is>
+      </c>
+      <c r="F67" t="inlineStr">
+        <is>
+          <t>M30</t>
+        </is>
+      </c>
+      <c r="G67" t="n">
+        <v>7503</v>
+      </c>
+      <c r="H67" t="inlineStr"/>
+      <c r="I67" t="n">
+        <v>0</v>
+      </c>
+      <c r="J67" t="n">
+        <v>7503</v>
+      </c>
+      <c r="K67" t="n">
+        <v>1</v>
+      </c>
+      <c r="L67" t="n">
+        <v>7503</v>
+      </c>
+      <c r="M67" t="inlineStr"/>
+      <c r="N67" t="inlineStr"/>
+      <c r="O67" t="n">
+        <v>0</v>
+      </c>
+      <c r="P67" t="inlineStr"/>
+      <c r="Q67" t="inlineStr"/>
+      <c r="R67" t="inlineStr">
+        <is>
+          <t>Mango Syrup</t>
+        </is>
+      </c>
+      <c r="S67" t="inlineStr">
+        <is>
+          <t>18 months</t>
+        </is>
+      </c>
+      <c r="T67" t="inlineStr">
+        <is>
+          <t>$15.60</t>
+        </is>
+      </c>
+      <c r="U67" t="n">
+        <v>2000</v>
+      </c>
+      <c r="V67" t="n">
+        <v>7503</v>
+      </c>
+    </row>
+    <row r="68">
+      <c r="A68" t="inlineStr">
+        <is>
+          <t>ZW01654</t>
+        </is>
+      </c>
+      <c r="B68" t="inlineStr">
+        <is>
+          <t>Thyme Japanese Cuisine</t>
+        </is>
+      </c>
+      <c r="C68" t="inlineStr">
+        <is>
+          <t>2026-07-01~2026-07-31</t>
+        </is>
+      </c>
+      <c r="D68" t="n">
+        <v>31</v>
+      </c>
+      <c r="E68" t="inlineStr">
+        <is>
+          <t>Testing Material 1</t>
+        </is>
+      </c>
+      <c r="F68" t="inlineStr">
+        <is>
+          <t>T01</t>
+        </is>
+      </c>
+      <c r="G68" t="n">
+        <v>0</v>
+      </c>
+      <c r="H68" t="inlineStr"/>
+      <c r="I68" t="n">
+        <v>0</v>
+      </c>
+      <c r="J68" t="n">
+        <v>0</v>
+      </c>
+      <c r="K68" t="n">
+        <v>1</v>
+      </c>
+      <c r="L68" t="n">
+        <v>0</v>
+      </c>
+      <c r="M68" t="inlineStr"/>
+      <c r="N68" t="inlineStr"/>
+      <c r="O68" t="n">
+        <v>0</v>
+      </c>
+      <c r="P68" t="inlineStr"/>
+      <c r="Q68" t="inlineStr"/>
+      <c r="R68" t="inlineStr">
+        <is>
+          <t>Testing Material 1</t>
+        </is>
+      </c>
+      <c r="S68" t="inlineStr"/>
+      <c r="T68" t="inlineStr"/>
+      <c r="U68" t="inlineStr"/>
+      <c r="V68" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="69">
+      <c r="A69" t="inlineStr">
+        <is>
+          <t>ZW01654</t>
+        </is>
+      </c>
+      <c r="B69" t="inlineStr">
+        <is>
+          <t>Thyme Japanese Cuisine</t>
+        </is>
+      </c>
+      <c r="C69" t="inlineStr">
+        <is>
+          <t>2026-07-01~2026-07-31</t>
+        </is>
+      </c>
+      <c r="D69" t="n">
+        <v>31</v>
+      </c>
+      <c r="E69" t="inlineStr">
+        <is>
+          <t>Testing Material 2</t>
+        </is>
+      </c>
+      <c r="F69" t="inlineStr">
+        <is>
+          <t>T02</t>
+        </is>
+      </c>
+      <c r="G69" t="n">
+        <v>0</v>
+      </c>
+      <c r="H69" t="inlineStr"/>
+      <c r="I69" t="n">
+        <v>0</v>
+      </c>
+      <c r="J69" t="n">
+        <v>0</v>
+      </c>
+      <c r="K69" t="n">
+        <v>1</v>
+      </c>
+      <c r="L69" t="n">
+        <v>0</v>
+      </c>
+      <c r="M69" t="inlineStr"/>
+      <c r="N69" t="inlineStr"/>
+      <c r="O69" t="n">
+        <v>0</v>
+      </c>
+      <c r="P69" t="inlineStr"/>
+      <c r="Q69" t="inlineStr"/>
+      <c r="R69" t="inlineStr">
+        <is>
+          <t>Testing Material 2</t>
+        </is>
+      </c>
+      <c r="S69" t="inlineStr"/>
+      <c r="T69" t="inlineStr"/>
+      <c r="U69" t="inlineStr"/>
+      <c r="V69" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="70">
+      <c r="A70" t="inlineStr">
+        <is>
+          <t>ZW01654</t>
+        </is>
+      </c>
+      <c r="B70" t="inlineStr">
+        <is>
+          <t>Thyme Japanese Cuisine</t>
+        </is>
+      </c>
+      <c r="C70" t="inlineStr">
+        <is>
+          <t>2026-07-01~2026-07-31</t>
+        </is>
+      </c>
+      <c r="D70" t="n">
+        <v>31</v>
+      </c>
+      <c r="E70" t="inlineStr">
+        <is>
+          <t>Testing Material 3</t>
+        </is>
+      </c>
+      <c r="F70" t="inlineStr">
+        <is>
+          <t>T03</t>
+        </is>
+      </c>
+      <c r="G70" t="n">
+        <v>0</v>
+      </c>
+      <c r="H70" t="inlineStr"/>
+      <c r="I70" t="n">
+        <v>0</v>
+      </c>
+      <c r="J70" t="n">
+        <v>0</v>
+      </c>
+      <c r="K70" t="n">
+        <v>1</v>
+      </c>
+      <c r="L70" t="n">
+        <v>0</v>
+      </c>
+      <c r="M70" t="inlineStr"/>
+      <c r="N70" t="inlineStr"/>
+      <c r="O70" t="n">
+        <v>0</v>
+      </c>
+      <c r="P70" t="inlineStr"/>
+      <c r="Q70" t="inlineStr"/>
+      <c r="R70" t="inlineStr">
+        <is>
+          <t>Testing Material 3</t>
+        </is>
+      </c>
+      <c r="S70" t="inlineStr"/>
+      <c r="T70" t="inlineStr"/>
+      <c r="U70" t="inlineStr"/>
+      <c r="V70" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="71">
+      <c r="A71" t="inlineStr">
+        <is>
+          <t>ZW01654</t>
+        </is>
+      </c>
+      <c r="B71" t="inlineStr">
+        <is>
+          <t>Thyme Japanese Cuisine</t>
+        </is>
+      </c>
+      <c r="C71" t="inlineStr">
+        <is>
+          <t>2026-07-01~2026-07-31</t>
+        </is>
+      </c>
+      <c r="D71" t="n">
+        <v>31</v>
+      </c>
+      <c r="E71" t="inlineStr">
+        <is>
+          <t>饮品奶油 BC01 Beverage Cream</t>
+        </is>
+      </c>
+      <c r="F71" t="inlineStr">
+        <is>
+          <t>M32</t>
+        </is>
+      </c>
+      <c r="G71" t="n">
+        <v>0</v>
+      </c>
+      <c r="H71" t="inlineStr"/>
+      <c r="I71" t="n">
+        <v>0</v>
+      </c>
+      <c r="J71" t="n">
+        <v>0</v>
+      </c>
+      <c r="K71" t="n">
+        <v>1</v>
+      </c>
+      <c r="L71" t="n">
+        <v>0</v>
+      </c>
+      <c r="M71" t="inlineStr"/>
+      <c r="N71" t="inlineStr"/>
+      <c r="O71" t="n">
+        <v>0</v>
+      </c>
+      <c r="P71" t="inlineStr"/>
+      <c r="Q71" t="inlineStr"/>
+      <c r="R71" t="inlineStr">
+        <is>
+          <t>BC01 Beverage Cream</t>
+        </is>
+      </c>
+      <c r="S71" t="inlineStr"/>
+      <c r="T71" t="inlineStr"/>
+      <c r="U71" t="inlineStr"/>
+      <c r="V71" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="72">
+      <c r="A72" t="inlineStr">
+        <is>
+          <t>ZW01654</t>
+        </is>
+      </c>
+      <c r="B72" t="inlineStr">
+        <is>
+          <t>Thyme Japanese Cuisine</t>
+        </is>
+      </c>
+      <c r="C72" t="inlineStr">
+        <is>
+          <t>2026-07-01~2026-07-31</t>
+        </is>
+      </c>
+      <c r="D72" t="n">
+        <v>31</v>
+      </c>
+      <c r="E72" t="inlineStr">
+        <is>
+          <t>Taro Syrup 鲜芋糖浆</t>
+        </is>
+      </c>
+      <c r="F72" t="inlineStr">
+        <is>
+          <t>T04</t>
+        </is>
+      </c>
+      <c r="G72" t="n">
+        <v>0</v>
+      </c>
+      <c r="H72" t="inlineStr"/>
+      <c r="I72" t="n">
+        <v>0</v>
+      </c>
+      <c r="J72" t="n">
+        <v>0</v>
+      </c>
+      <c r="K72" t="n">
+        <v>1</v>
+      </c>
+      <c r="L72" t="n">
+        <v>0</v>
+      </c>
+      <c r="M72" t="inlineStr"/>
+      <c r="N72" t="inlineStr"/>
+      <c r="O72" t="n">
+        <v>0</v>
+      </c>
+      <c r="P72" t="inlineStr"/>
+      <c r="Q72" t="inlineStr"/>
+      <c r="R72" t="inlineStr">
+        <is>
+          <t>Taro Syrup</t>
+        </is>
+      </c>
+      <c r="S72" t="inlineStr"/>
+      <c r="T72" t="inlineStr"/>
+      <c r="U72" t="inlineStr"/>
+      <c r="V72" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="73">
+      <c r="A73" t="inlineStr">
+        <is>
+          <t>ZW01654</t>
+        </is>
+      </c>
+      <c r="B73" t="inlineStr">
+        <is>
+          <t>Thyme Japanese Cuisine</t>
+        </is>
+      </c>
+      <c r="C73" t="inlineStr">
+        <is>
+          <t>2026-07-01~2026-07-31</t>
+        </is>
+      </c>
+      <c r="D73" t="n">
+        <v>31</v>
+      </c>
+      <c r="E73" t="inlineStr">
+        <is>
+          <t>Watermelon Syrup</t>
+        </is>
+      </c>
+      <c r="F73" t="inlineStr">
+        <is>
+          <t>M31</t>
+        </is>
+      </c>
+      <c r="G73" t="n">
+        <v>0</v>
+      </c>
+      <c r="H73" t="inlineStr"/>
+      <c r="I73" t="n">
+        <v>0</v>
+      </c>
+      <c r="J73" t="n">
+        <v>0</v>
+      </c>
+      <c r="K73" t="n">
+        <v>1</v>
+      </c>
+      <c r="L73" t="n">
+        <v>0</v>
+      </c>
+      <c r="M73" t="inlineStr"/>
+      <c r="N73" t="inlineStr"/>
+      <c r="O73" t="n">
+        <v>0</v>
+      </c>
+      <c r="P73" t="inlineStr"/>
+      <c r="Q73" t="inlineStr"/>
+      <c r="R73" t="inlineStr">
+        <is>
+          <t>Watermelon Syrup</t>
+        </is>
+      </c>
+      <c r="S73" t="inlineStr"/>
+      <c r="T73" t="inlineStr"/>
+      <c r="U73" t="inlineStr"/>
+      <c r="V73" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="74">
+      <c r="A74" t="inlineStr">
+        <is>
+          <t>ZW01654</t>
+        </is>
+      </c>
+      <c r="B74" t="inlineStr">
+        <is>
+          <t>Thyme Japanese Cuisine</t>
+        </is>
+      </c>
+      <c r="C74" t="inlineStr">
+        <is>
+          <t>2026-07-01~2026-07-31</t>
+        </is>
+      </c>
+      <c r="D74" t="n">
+        <v>31</v>
+      </c>
+      <c r="E74" t="inlineStr">
+        <is>
+          <t>Orange Syrup</t>
+        </is>
+      </c>
+      <c r="F74" t="inlineStr">
+        <is>
+          <t>M33</t>
+        </is>
+      </c>
+      <c r="G74" t="n">
+        <v>0</v>
+      </c>
+      <c r="H74" t="inlineStr"/>
+      <c r="I74" t="n">
+        <v>0</v>
+      </c>
+      <c r="J74" t="n">
+        <v>0</v>
+      </c>
+      <c r="K74" t="n">
+        <v>1</v>
+      </c>
+      <c r="L74" t="n">
+        <v>0</v>
+      </c>
+      <c r="M74" t="inlineStr"/>
+      <c r="N74" t="inlineStr"/>
+      <c r="O74" t="n">
+        <v>0</v>
+      </c>
+      <c r="P74" t="inlineStr"/>
+      <c r="Q74" t="inlineStr"/>
+      <c r="R74" t="inlineStr">
+        <is>
+          <t>Orange Syrup</t>
+        </is>
+      </c>
+      <c r="S74" t="inlineStr"/>
+      <c r="T74" t="inlineStr"/>
+      <c r="U74" t="inlineStr"/>
+      <c r="V74" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="75">
+      <c r="A75" t="inlineStr">
+        <is>
+          <t>ZW01654</t>
+        </is>
+      </c>
+      <c r="B75" t="inlineStr">
+        <is>
+          <t>Thyme Japanese Cuisine</t>
+        </is>
+      </c>
+      <c r="C75" t="inlineStr">
+        <is>
+          <t>2026-07-01~2026-07-31</t>
+        </is>
+      </c>
+      <c r="D75" t="n">
+        <v>31</v>
+      </c>
+      <c r="E75" t="inlineStr">
+        <is>
+          <t>Passion Fruit Syrup</t>
+        </is>
+      </c>
+      <c r="F75" t="inlineStr">
+        <is>
+          <t>M34</t>
+        </is>
+      </c>
+      <c r="G75" t="n">
+        <v>0</v>
+      </c>
+      <c r="H75" t="inlineStr"/>
+      <c r="I75" t="n">
+        <v>0</v>
+      </c>
+      <c r="J75" t="n">
+        <v>0</v>
+      </c>
+      <c r="K75" t="n">
+        <v>1</v>
+      </c>
+      <c r="L75" t="n">
+        <v>0</v>
+      </c>
+      <c r="M75" t="inlineStr"/>
+      <c r="N75" t="inlineStr"/>
+      <c r="O75" t="n">
+        <v>0</v>
+      </c>
+      <c r="P75" t="inlineStr"/>
+      <c r="Q75" t="inlineStr"/>
+      <c r="R75" t="inlineStr">
+        <is>
+          <t>Passion Fruit Syrup</t>
+        </is>
+      </c>
+      <c r="S75" t="inlineStr"/>
+      <c r="T75" t="inlineStr"/>
+      <c r="U75" t="inlineStr"/>
+      <c r="V75" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="76">
+      <c r="A76" t="inlineStr">
+        <is>
+          <t>ZW01654</t>
+        </is>
+      </c>
+      <c r="B76" t="inlineStr">
+        <is>
+          <t>Thyme Japanese Cuisine</t>
+        </is>
+      </c>
+      <c r="C76" t="inlineStr">
+        <is>
+          <t>2026-07-01~2026-07-31</t>
+        </is>
+      </c>
+      <c r="D76" t="n">
+        <v>31</v>
+      </c>
+      <c r="E76" t="inlineStr">
+        <is>
+          <t>全脂牛奶 Whole Milk</t>
+        </is>
+      </c>
+      <c r="F76" t="inlineStr">
+        <is>
+          <t>M35</t>
+        </is>
+      </c>
+      <c r="G76" t="n">
+        <v>0</v>
+      </c>
+      <c r="H76" t="inlineStr"/>
+      <c r="I76" t="n">
+        <v>0</v>
+      </c>
+      <c r="J76" t="n">
+        <v>0</v>
+      </c>
+      <c r="K76" t="n">
+        <v>1</v>
+      </c>
+      <c r="L76" t="n">
+        <v>0</v>
+      </c>
+      <c r="M76" t="inlineStr"/>
+      <c r="N76" t="inlineStr"/>
+      <c r="O76" t="n">
+        <v>0</v>
+      </c>
+      <c r="P76" t="inlineStr"/>
+      <c r="Q76" t="inlineStr"/>
+      <c r="R76" t="inlineStr">
+        <is>
+          <t>Whole Milk</t>
+        </is>
+      </c>
+      <c r="S76" t="inlineStr"/>
+      <c r="T76" t="inlineStr"/>
+      <c r="U76" t="inlineStr"/>
+      <c r="V76" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="77">
+      <c r="A77" t="inlineStr">
+        <is>
+          <t>ZW01654</t>
+        </is>
+      </c>
+      <c r="B77" t="inlineStr">
+        <is>
+          <t>Thyme Japanese Cuisine</t>
+        </is>
+      </c>
+      <c r="C77" t="inlineStr">
+        <is>
+          <t>2026-07-01~2026-07-31</t>
+        </is>
+      </c>
+      <c r="D77" t="n">
+        <v>31</v>
+      </c>
+      <c r="E77" t="inlineStr">
+        <is>
+          <t>石榴糖浆 Pomegranate Syrup</t>
+        </is>
+      </c>
+      <c r="F77" t="inlineStr">
+        <is>
+          <t>MT14</t>
+        </is>
+      </c>
+      <c r="G77" t="n">
+        <v>0</v>
+      </c>
+      <c r="H77" t="inlineStr"/>
+      <c r="I77" t="n">
+        <v>0</v>
+      </c>
+      <c r="J77" t="n">
+        <v>0</v>
+      </c>
+      <c r="K77" t="n">
+        <v>1</v>
+      </c>
+      <c r="L77" t="n">
+        <v>0</v>
+      </c>
+      <c r="M77" t="inlineStr"/>
+      <c r="N77" t="inlineStr"/>
+      <c r="O77" t="n">
+        <v>0</v>
+      </c>
+      <c r="P77" t="inlineStr"/>
+      <c r="Q77" t="inlineStr"/>
+      <c r="R77" t="inlineStr">
+        <is>
+          <t>Pomegranate Syrup</t>
+        </is>
+      </c>
+      <c r="S77" t="inlineStr"/>
+      <c r="T77" t="inlineStr"/>
+      <c r="U77" t="inlineStr"/>
+      <c r="V77" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="78">
+      <c r="A78" t="inlineStr">
+        <is>
+          <t>ZW02551</t>
+        </is>
+      </c>
+      <c r="B78" t="inlineStr">
+        <is>
+          <t>HQ Woburn</t>
+        </is>
+      </c>
+      <c r="C78" t="inlineStr">
+        <is>
+          <t>2026-07-01~2026-07-31</t>
+        </is>
+      </c>
+      <c r="D78" t="n">
+        <v>31</v>
+      </c>
+      <c r="E78" t="inlineStr">
+        <is>
+          <t>冰糖糖浆 Fructose Syrup</t>
+        </is>
+      </c>
+      <c r="F78" t="inlineStr">
+        <is>
+          <t>M13</t>
+        </is>
+      </c>
+      <c r="G78" t="n">
+        <v>1076</v>
+      </c>
+      <c r="H78" t="inlineStr"/>
+      <c r="I78" t="n">
+        <v>0</v>
+      </c>
+      <c r="J78" t="n">
+        <v>1076</v>
+      </c>
+      <c r="K78" t="n">
+        <v>1</v>
+      </c>
+      <c r="L78" t="n">
+        <v>1076</v>
+      </c>
+      <c r="M78" t="inlineStr"/>
+      <c r="N78" t="inlineStr"/>
+      <c r="O78" t="n">
+        <v>0</v>
+      </c>
+      <c r="P78" t="inlineStr"/>
+      <c r="Q78" t="inlineStr"/>
+      <c r="R78" t="inlineStr">
+        <is>
+          <t>Fructose Syrup</t>
+        </is>
+      </c>
+      <c r="S78" t="inlineStr">
+        <is>
+          <t>18 months</t>
+        </is>
+      </c>
+      <c r="T78" t="inlineStr">
+        <is>
+          <t>$15.60</t>
+        </is>
+      </c>
+      <c r="U78" t="n">
+        <v>2000</v>
+      </c>
+      <c r="V78" t="n">
+        <v>1076</v>
+      </c>
+    </row>
+    <row r="79">
+      <c r="A79" t="inlineStr">
+        <is>
+          <t>ZW02551</t>
+        </is>
+      </c>
+      <c r="B79" t="inlineStr">
+        <is>
+          <t>HQ Woburn</t>
+        </is>
+      </c>
+      <c r="C79" t="inlineStr">
+        <is>
+          <t>2026-07-01~2026-07-31</t>
+        </is>
+      </c>
+      <c r="D79" t="n">
+        <v>31</v>
+      </c>
+      <c r="E79" t="inlineStr">
+        <is>
+          <t>冰勃朗 Ice Blanc</t>
+        </is>
+      </c>
+      <c r="F79" t="inlineStr">
+        <is>
+          <t>M14</t>
+        </is>
+      </c>
+      <c r="G79" t="n">
+        <v>1432</v>
+      </c>
+      <c r="H79" t="inlineStr"/>
+      <c r="I79" t="n">
+        <v>0</v>
+      </c>
+      <c r="J79" t="n">
+        <v>1432</v>
+      </c>
+      <c r="K79" t="n">
+        <v>1</v>
+      </c>
+      <c r="L79" t="n">
+        <v>1432</v>
+      </c>
+      <c r="M79" t="inlineStr"/>
+      <c r="N79" t="inlineStr"/>
+      <c r="O79" t="n">
+        <v>0</v>
+      </c>
+      <c r="P79" t="inlineStr"/>
+      <c r="Q79" t="inlineStr"/>
+      <c r="R79" t="inlineStr">
+        <is>
+          <t>Ice Blanc</t>
+        </is>
+      </c>
+      <c r="S79" t="inlineStr">
+        <is>
+          <t>9 months</t>
+        </is>
+      </c>
+      <c r="T79" t="inlineStr">
+        <is>
+          <t>$12.00</t>
+        </is>
+      </c>
+      <c r="U79" t="n">
+        <v>1000</v>
+      </c>
+      <c r="V79" t="n">
+        <v>1432</v>
+      </c>
+    </row>
+    <row r="80">
+      <c r="A80" t="inlineStr">
+        <is>
+          <t>ZW02551</t>
+        </is>
+      </c>
+      <c r="B80" t="inlineStr">
+        <is>
+          <t>HQ Woburn</t>
+        </is>
+      </c>
+      <c r="C80" t="inlineStr">
+        <is>
+          <t>2026-07-01~2026-07-31</t>
+        </is>
+      </c>
+      <c r="D80" t="n">
+        <v>31</v>
+      </c>
+      <c r="E80" t="inlineStr">
+        <is>
+          <t>锡兰红茶茶汤 Black Tea</t>
+        </is>
+      </c>
+      <c r="F80" t="inlineStr">
+        <is>
+          <t>M16</t>
+        </is>
+      </c>
+      <c r="G80" t="n">
+        <v>4227</v>
+      </c>
+      <c r="H80" t="inlineStr"/>
+      <c r="I80" t="n">
+        <v>0</v>
+      </c>
+      <c r="J80" t="n">
+        <v>4227</v>
+      </c>
+      <c r="K80" t="n">
+        <v>1</v>
+      </c>
+      <c r="L80" t="n">
+        <v>4227</v>
+      </c>
+      <c r="M80" t="inlineStr"/>
+      <c r="N80" t="inlineStr"/>
+      <c r="O80" t="n">
+        <v>0</v>
+      </c>
+      <c r="P80" t="inlineStr"/>
+      <c r="Q80" t="inlineStr"/>
+      <c r="R80" t="inlineStr">
+        <is>
+          <t>Black Tea</t>
+        </is>
+      </c>
+      <c r="S80" t="inlineStr">
+        <is>
+          <t>24 months</t>
+        </is>
+      </c>
+      <c r="T80" t="inlineStr">
+        <is>
+          <t>$12.30</t>
+        </is>
+      </c>
+      <c r="U80" t="n">
+        <v>500</v>
+      </c>
+      <c r="V80" t="n">
+        <v>126.81</v>
+      </c>
+    </row>
+    <row r="81">
+      <c r="A81" t="inlineStr">
+        <is>
+          <t>ZW02551</t>
+        </is>
+      </c>
+      <c r="B81" t="inlineStr">
+        <is>
+          <t>HQ Woburn</t>
+        </is>
+      </c>
+      <c r="C81" t="inlineStr">
+        <is>
+          <t>2026-07-01~2026-07-31</t>
+        </is>
+      </c>
+      <c r="D81" t="n">
+        <v>31</v>
+      </c>
+      <c r="E81" t="inlineStr">
+        <is>
+          <t>冰水 Cold Water</t>
+        </is>
+      </c>
+      <c r="F81" t="inlineStr">
+        <is>
+          <t>M22</t>
+        </is>
+      </c>
+      <c r="G81" t="n">
+        <v>5954</v>
+      </c>
+      <c r="H81" t="inlineStr"/>
+      <c r="I81" t="n">
+        <v>0</v>
+      </c>
+      <c r="J81" t="n">
+        <v>5954</v>
+      </c>
+      <c r="K81" t="n">
+        <v>1</v>
+      </c>
+      <c r="L81" t="n">
+        <v>5954</v>
+      </c>
+      <c r="M81" t="inlineStr"/>
+      <c r="N81" t="inlineStr"/>
+      <c r="O81" t="n">
+        <v>0</v>
+      </c>
+      <c r="P81" t="inlineStr"/>
+      <c r="Q81" t="inlineStr"/>
+      <c r="R81" t="inlineStr">
+        <is>
+          <t>Cold Water</t>
+        </is>
+      </c>
+      <c r="S81" t="inlineStr"/>
+      <c r="T81" t="inlineStr"/>
+      <c r="U81" t="inlineStr"/>
+      <c r="V81" t="n">
+        <v>5954</v>
+      </c>
+    </row>
+    <row r="82">
+      <c r="A82" t="inlineStr">
+        <is>
+          <t>ZW02551</t>
+        </is>
+      </c>
+      <c r="B82" t="inlineStr">
+        <is>
+          <t>HQ Woburn</t>
+        </is>
+      </c>
+      <c r="C82" t="inlineStr">
+        <is>
+          <t>2026-07-01~2026-07-31</t>
+        </is>
+      </c>
+      <c r="D82" t="n">
+        <v>31</v>
+      </c>
+      <c r="E82" t="inlineStr">
+        <is>
+          <t>茉莉雪芽茶汤 Green Tea</t>
+        </is>
+      </c>
+      <c r="F82" t="inlineStr">
+        <is>
+          <t>M23</t>
+        </is>
+      </c>
+      <c r="G82" t="n">
+        <v>2623</v>
+      </c>
+      <c r="H82" t="inlineStr"/>
+      <c r="I82" t="n">
+        <v>0</v>
+      </c>
+      <c r="J82" t="n">
+        <v>2623</v>
+      </c>
+      <c r="K82" t="n">
+        <v>1</v>
+      </c>
+      <c r="L82" t="n">
+        <v>2623</v>
+      </c>
+      <c r="M82" t="inlineStr"/>
+      <c r="N82" t="inlineStr"/>
+      <c r="O82" t="n">
+        <v>0</v>
+      </c>
+      <c r="P82" t="inlineStr"/>
+      <c r="Q82" t="inlineStr"/>
+      <c r="R82" t="inlineStr">
+        <is>
+          <t>Green Tea</t>
+        </is>
+      </c>
+      <c r="S82" t="inlineStr">
+        <is>
+          <t>24 months</t>
+        </is>
+      </c>
+      <c r="T82" t="inlineStr">
+        <is>
+          <t>$16.20</t>
+        </is>
+      </c>
+      <c r="U82" t="n">
+        <v>500</v>
+      </c>
+      <c r="V82" t="n">
+        <v>78.69</v>
+      </c>
+    </row>
+    <row r="83">
+      <c r="A83" t="inlineStr">
+        <is>
+          <t>ZW02551</t>
+        </is>
+      </c>
+      <c r="B83" t="inlineStr">
+        <is>
+          <t>HQ Woburn</t>
+        </is>
+      </c>
+      <c r="C83" t="inlineStr">
+        <is>
+          <t>2026-07-01~2026-07-31</t>
+        </is>
+      </c>
+      <c r="D83" t="n">
+        <v>31</v>
+      </c>
+      <c r="E83" t="inlineStr">
+        <is>
+          <t>黑糖糖浆 Brown Sugar</t>
+        </is>
+      </c>
+      <c r="F83" t="inlineStr">
+        <is>
+          <t>M27</t>
+        </is>
+      </c>
+      <c r="G83" t="n">
+        <v>1420</v>
+      </c>
+      <c r="H83" t="inlineStr"/>
+      <c r="I83" t="n">
+        <v>0</v>
+      </c>
+      <c r="J83" t="n">
+        <v>1420</v>
+      </c>
+      <c r="K83" t="n">
+        <v>1</v>
+      </c>
+      <c r="L83" t="n">
+        <v>1420</v>
+      </c>
+      <c r="M83" t="inlineStr"/>
+      <c r="N83" t="inlineStr"/>
+      <c r="O83" t="n">
+        <v>0</v>
+      </c>
+      <c r="P83" t="inlineStr"/>
+      <c r="Q83" t="inlineStr"/>
+      <c r="R83" t="inlineStr">
+        <is>
+          <t>Brown Sugar</t>
+        </is>
+      </c>
+      <c r="S83" t="inlineStr">
+        <is>
+          <t>18 months</t>
+        </is>
+      </c>
+      <c r="T83" t="inlineStr">
+        <is>
+          <t>$15.60</t>
+        </is>
+      </c>
+      <c r="U83" t="n">
+        <v>2000</v>
+      </c>
+      <c r="V83" t="n">
+        <v>1420</v>
+      </c>
+    </row>
+    <row r="84">
+      <c r="A84" t="inlineStr">
+        <is>
+          <t>ZW02551</t>
+        </is>
+      </c>
+      <c r="B84" t="inlineStr">
+        <is>
+          <t>HQ Woburn</t>
+        </is>
+      </c>
+      <c r="C84" t="inlineStr">
+        <is>
+          <t>2026-07-01~2026-07-31</t>
+        </is>
+      </c>
+      <c r="D84" t="n">
+        <v>31</v>
+      </c>
+      <c r="E84" t="inlineStr">
+        <is>
+          <t>蜜桃糖浆 Peach Syrup</t>
+        </is>
+      </c>
+      <c r="F84" t="inlineStr">
+        <is>
+          <t>M28</t>
+        </is>
+      </c>
+      <c r="G84" t="n">
+        <v>495</v>
+      </c>
+      <c r="H84" t="inlineStr"/>
+      <c r="I84" t="n">
+        <v>0</v>
+      </c>
+      <c r="J84" t="n">
+        <v>495</v>
+      </c>
+      <c r="K84" t="n">
+        <v>1</v>
+      </c>
+      <c r="L84" t="n">
+        <v>495</v>
+      </c>
+      <c r="M84" t="inlineStr"/>
+      <c r="N84" t="inlineStr"/>
+      <c r="O84" t="n">
+        <v>0</v>
+      </c>
+      <c r="P84" t="inlineStr"/>
+      <c r="Q84" t="inlineStr"/>
+      <c r="R84" t="inlineStr">
+        <is>
+          <t>Peach Syrup</t>
+        </is>
+      </c>
+      <c r="S84" t="inlineStr">
+        <is>
+          <t>18 months</t>
+        </is>
+      </c>
+      <c r="T84" t="inlineStr">
+        <is>
+          <t>$16.80</t>
+        </is>
+      </c>
+      <c r="U84" t="n">
+        <v>2000</v>
+      </c>
+      <c r="V84" t="n">
+        <v>495</v>
+      </c>
+    </row>
+    <row r="85">
+      <c r="A85" t="inlineStr">
+        <is>
+          <t>ZW02551</t>
+        </is>
+      </c>
+      <c r="B85" t="inlineStr">
+        <is>
+          <t>HQ Woburn</t>
+        </is>
+      </c>
+      <c r="C85" t="inlineStr">
+        <is>
+          <t>2026-07-01~2026-07-31</t>
+        </is>
+      </c>
+      <c r="D85" t="n">
+        <v>31</v>
+      </c>
+      <c r="E85" t="inlineStr">
+        <is>
+          <t>荔枝糖浆 Lychee Syrup</t>
+        </is>
+      </c>
+      <c r="F85" t="inlineStr">
+        <is>
+          <t>M29</t>
+        </is>
+      </c>
+      <c r="G85" t="n">
+        <v>0</v>
+      </c>
+      <c r="H85" t="inlineStr"/>
+      <c r="I85" t="n">
+        <v>0</v>
+      </c>
+      <c r="J85" t="n">
+        <v>0</v>
+      </c>
+      <c r="K85" t="n">
+        <v>1</v>
+      </c>
+      <c r="L85" t="n">
+        <v>0</v>
+      </c>
+      <c r="M85" t="inlineStr"/>
+      <c r="N85" t="inlineStr"/>
+      <c r="O85" t="n">
+        <v>0</v>
+      </c>
+      <c r="P85" t="inlineStr"/>
+      <c r="Q85" t="inlineStr"/>
+      <c r="R85" t="inlineStr">
+        <is>
+          <t>Lychee Syrup</t>
+        </is>
+      </c>
+      <c r="S85" t="inlineStr"/>
+      <c r="T85" t="inlineStr"/>
+      <c r="U85" t="inlineStr"/>
+      <c r="V85" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="86">
+      <c r="A86" t="inlineStr">
+        <is>
+          <t>ZW02551</t>
+        </is>
+      </c>
+      <c r="B86" t="inlineStr">
+        <is>
+          <t>HQ Woburn</t>
+        </is>
+      </c>
+      <c r="C86" t="inlineStr">
+        <is>
+          <t>2026-07-01~2026-07-31</t>
+        </is>
+      </c>
+      <c r="D86" t="n">
+        <v>31</v>
+      </c>
+      <c r="E86" t="inlineStr">
+        <is>
+          <t>芒果糖浆 Mango Syrup</t>
+        </is>
+      </c>
+      <c r="F86" t="inlineStr">
+        <is>
+          <t>M30</t>
+        </is>
+      </c>
+      <c r="G86" t="n">
+        <v>550</v>
+      </c>
+      <c r="H86" t="inlineStr"/>
+      <c r="I86" t="n">
+        <v>0</v>
+      </c>
+      <c r="J86" t="n">
+        <v>550</v>
+      </c>
+      <c r="K86" t="n">
+        <v>1</v>
+      </c>
+      <c r="L86" t="n">
+        <v>550</v>
+      </c>
+      <c r="M86" t="inlineStr"/>
+      <c r="N86" t="inlineStr"/>
+      <c r="O86" t="n">
+        <v>0</v>
+      </c>
+      <c r="P86" t="inlineStr"/>
+      <c r="Q86" t="inlineStr"/>
+      <c r="R86" t="inlineStr">
+        <is>
+          <t>Mango Syrup</t>
+        </is>
+      </c>
+      <c r="S86" t="inlineStr">
+        <is>
+          <t>18 months</t>
+        </is>
+      </c>
+      <c r="T86" t="inlineStr">
+        <is>
+          <t>$15.60</t>
+        </is>
+      </c>
+      <c r="U86" t="n">
+        <v>2000</v>
+      </c>
+      <c r="V86" t="n">
+        <v>550</v>
+      </c>
+    </row>
+    <row r="87">
+      <c r="A87" t="inlineStr">
+        <is>
+          <t>ZW02551</t>
+        </is>
+      </c>
+      <c r="B87" t="inlineStr">
+        <is>
+          <t>HQ Woburn</t>
+        </is>
+      </c>
+      <c r="C87" t="inlineStr">
+        <is>
+          <t>2026-07-01~2026-07-31</t>
+        </is>
+      </c>
+      <c r="D87" t="n">
+        <v>31</v>
+      </c>
+      <c r="E87" t="inlineStr">
+        <is>
+          <t>Testing Material 1</t>
+        </is>
+      </c>
+      <c r="F87" t="inlineStr">
+        <is>
+          <t>T01</t>
+        </is>
+      </c>
+      <c r="G87" t="n">
+        <v>0</v>
+      </c>
+      <c r="H87" t="inlineStr"/>
+      <c r="I87" t="n">
+        <v>0</v>
+      </c>
+      <c r="J87" t="n">
+        <v>0</v>
+      </c>
+      <c r="K87" t="n">
+        <v>1</v>
+      </c>
+      <c r="L87" t="n">
+        <v>0</v>
+      </c>
+      <c r="M87" t="inlineStr"/>
+      <c r="N87" t="inlineStr"/>
+      <c r="O87" t="n">
+        <v>0</v>
+      </c>
+      <c r="P87" t="inlineStr"/>
+      <c r="Q87" t="inlineStr"/>
+      <c r="R87" t="inlineStr">
+        <is>
+          <t>Testing Material 1</t>
+        </is>
+      </c>
+      <c r="S87" t="inlineStr"/>
+      <c r="T87" t="inlineStr"/>
+      <c r="U87" t="inlineStr"/>
+      <c r="V87" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="88">
+      <c r="A88" t="inlineStr">
+        <is>
+          <t>ZW02551</t>
+        </is>
+      </c>
+      <c r="B88" t="inlineStr">
+        <is>
+          <t>HQ Woburn</t>
+        </is>
+      </c>
+      <c r="C88" t="inlineStr">
+        <is>
+          <t>2026-07-01~2026-07-31</t>
+        </is>
+      </c>
+      <c r="D88" t="n">
+        <v>31</v>
+      </c>
+      <c r="E88" t="inlineStr">
+        <is>
+          <t>Testing Material 2</t>
+        </is>
+      </c>
+      <c r="F88" t="inlineStr">
+        <is>
+          <t>T02</t>
+        </is>
+      </c>
+      <c r="G88" t="n">
+        <v>0</v>
+      </c>
+      <c r="H88" t="inlineStr"/>
+      <c r="I88" t="n">
+        <v>0</v>
+      </c>
+      <c r="J88" t="n">
+        <v>0</v>
+      </c>
+      <c r="K88" t="n">
+        <v>1</v>
+      </c>
+      <c r="L88" t="n">
+        <v>0</v>
+      </c>
+      <c r="M88" t="inlineStr"/>
+      <c r="N88" t="inlineStr"/>
+      <c r="O88" t="n">
+        <v>0</v>
+      </c>
+      <c r="P88" t="inlineStr"/>
+      <c r="Q88" t="inlineStr"/>
+      <c r="R88" t="inlineStr">
+        <is>
+          <t>Testing Material 2</t>
+        </is>
+      </c>
+      <c r="S88" t="inlineStr"/>
+      <c r="T88" t="inlineStr"/>
+      <c r="U88" t="inlineStr"/>
+      <c r="V88" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="89">
+      <c r="A89" t="inlineStr">
+        <is>
+          <t>ZW02551</t>
+        </is>
+      </c>
+      <c r="B89" t="inlineStr">
+        <is>
+          <t>HQ Woburn</t>
+        </is>
+      </c>
+      <c r="C89" t="inlineStr">
+        <is>
+          <t>2026-07-01~2026-07-31</t>
+        </is>
+      </c>
+      <c r="D89" t="n">
+        <v>31</v>
+      </c>
+      <c r="E89" t="inlineStr">
+        <is>
+          <t>Testing Material 3</t>
+        </is>
+      </c>
+      <c r="F89" t="inlineStr">
+        <is>
+          <t>T03</t>
+        </is>
+      </c>
+      <c r="G89" t="n">
+        <v>0</v>
+      </c>
+      <c r="H89" t="inlineStr"/>
+      <c r="I89" t="n">
+        <v>0</v>
+      </c>
+      <c r="J89" t="n">
+        <v>0</v>
+      </c>
+      <c r="K89" t="n">
+        <v>1</v>
+      </c>
+      <c r="L89" t="n">
+        <v>0</v>
+      </c>
+      <c r="M89" t="inlineStr"/>
+      <c r="N89" t="inlineStr"/>
+      <c r="O89" t="n">
+        <v>0</v>
+      </c>
+      <c r="P89" t="inlineStr"/>
+      <c r="Q89" t="inlineStr"/>
+      <c r="R89" t="inlineStr">
+        <is>
+          <t>Testing Material 3</t>
+        </is>
+      </c>
+      <c r="S89" t="inlineStr"/>
+      <c r="T89" t="inlineStr"/>
+      <c r="U89" t="inlineStr"/>
+      <c r="V89" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="90">
+      <c r="A90" t="inlineStr">
+        <is>
+          <t>ZW02551</t>
+        </is>
+      </c>
+      <c r="B90" t="inlineStr">
+        <is>
+          <t>HQ Woburn</t>
+        </is>
+      </c>
+      <c r="C90" t="inlineStr">
+        <is>
+          <t>2026-07-01~2026-07-31</t>
+        </is>
+      </c>
+      <c r="D90" t="n">
+        <v>31</v>
+      </c>
+      <c r="E90" t="inlineStr">
+        <is>
+          <t>饮品奶油 BC01 Beverage Cream</t>
+        </is>
+      </c>
+      <c r="F90" t="inlineStr">
+        <is>
+          <t>M32</t>
+        </is>
+      </c>
+      <c r="G90" t="n">
+        <v>0</v>
+      </c>
+      <c r="H90" t="inlineStr"/>
+      <c r="I90" t="n">
+        <v>0</v>
+      </c>
+      <c r="J90" t="n">
+        <v>0</v>
+      </c>
+      <c r="K90" t="n">
+        <v>1</v>
+      </c>
+      <c r="L90" t="n">
+        <v>0</v>
+      </c>
+      <c r="M90" t="inlineStr"/>
+      <c r="N90" t="inlineStr"/>
+      <c r="O90" t="n">
+        <v>0</v>
+      </c>
+      <c r="P90" t="inlineStr"/>
+      <c r="Q90" t="inlineStr"/>
+      <c r="R90" t="inlineStr">
+        <is>
+          <t>BC01 Beverage Cream</t>
+        </is>
+      </c>
+      <c r="S90" t="inlineStr"/>
+      <c r="T90" t="inlineStr"/>
+      <c r="U90" t="inlineStr"/>
+      <c r="V90" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="91">
+      <c r="A91" t="inlineStr">
+        <is>
+          <t>ZW02551</t>
+        </is>
+      </c>
+      <c r="B91" t="inlineStr">
+        <is>
+          <t>HQ Woburn</t>
+        </is>
+      </c>
+      <c r="C91" t="inlineStr">
+        <is>
+          <t>2026-07-01~2026-07-31</t>
+        </is>
+      </c>
+      <c r="D91" t="n">
+        <v>31</v>
+      </c>
+      <c r="E91" t="inlineStr">
+        <is>
+          <t>Taro Syrup 鲜芋糖浆</t>
+        </is>
+      </c>
+      <c r="F91" t="inlineStr">
+        <is>
+          <t>T04</t>
+        </is>
+      </c>
+      <c r="G91" t="n">
+        <v>0</v>
+      </c>
+      <c r="H91" t="inlineStr"/>
+      <c r="I91" t="n">
+        <v>0</v>
+      </c>
+      <c r="J91" t="n">
+        <v>0</v>
+      </c>
+      <c r="K91" t="n">
+        <v>1</v>
+      </c>
+      <c r="L91" t="n">
+        <v>0</v>
+      </c>
+      <c r="M91" t="inlineStr"/>
+      <c r="N91" t="inlineStr"/>
+      <c r="O91" t="n">
+        <v>0</v>
+      </c>
+      <c r="P91" t="inlineStr"/>
+      <c r="Q91" t="inlineStr"/>
+      <c r="R91" t="inlineStr">
+        <is>
+          <t>Taro Syrup</t>
+        </is>
+      </c>
+      <c r="S91" t="inlineStr"/>
+      <c r="T91" t="inlineStr"/>
+      <c r="U91" t="inlineStr"/>
+      <c r="V91" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="92">
+      <c r="A92" t="inlineStr">
+        <is>
+          <t>ZW02551</t>
+        </is>
+      </c>
+      <c r="B92" t="inlineStr">
+        <is>
+          <t>HQ Woburn</t>
+        </is>
+      </c>
+      <c r="C92" t="inlineStr">
+        <is>
+          <t>2026-07-01~2026-07-31</t>
+        </is>
+      </c>
+      <c r="D92" t="n">
+        <v>31</v>
+      </c>
+      <c r="E92" t="inlineStr">
+        <is>
+          <t>Watermelon Syrup</t>
+        </is>
+      </c>
+      <c r="F92" t="inlineStr">
+        <is>
+          <t>M31</t>
+        </is>
+      </c>
+      <c r="G92" t="n">
+        <v>0</v>
+      </c>
+      <c r="H92" t="inlineStr"/>
+      <c r="I92" t="n">
+        <v>0</v>
+      </c>
+      <c r="J92" t="n">
+        <v>0</v>
+      </c>
+      <c r="K92" t="n">
+        <v>1</v>
+      </c>
+      <c r="L92" t="n">
+        <v>0</v>
+      </c>
+      <c r="M92" t="inlineStr"/>
+      <c r="N92" t="inlineStr"/>
+      <c r="O92" t="n">
+        <v>0</v>
+      </c>
+      <c r="P92" t="inlineStr"/>
+      <c r="Q92" t="inlineStr"/>
+      <c r="R92" t="inlineStr">
+        <is>
+          <t>Watermelon Syrup</t>
+        </is>
+      </c>
+      <c r="S92" t="inlineStr"/>
+      <c r="T92" t="inlineStr"/>
+      <c r="U92" t="inlineStr"/>
+      <c r="V92" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="93">
+      <c r="A93" t="inlineStr">
+        <is>
+          <t>ZW02551</t>
+        </is>
+      </c>
+      <c r="B93" t="inlineStr">
+        <is>
+          <t>HQ Woburn</t>
+        </is>
+      </c>
+      <c r="C93" t="inlineStr">
+        <is>
+          <t>2026-07-01~2026-07-31</t>
+        </is>
+      </c>
+      <c r="D93" t="n">
+        <v>31</v>
+      </c>
+      <c r="E93" t="inlineStr">
+        <is>
+          <t>Orange Syrup</t>
+        </is>
+      </c>
+      <c r="F93" t="inlineStr">
+        <is>
+          <t>M33</t>
+        </is>
+      </c>
+      <c r="G93" t="n">
+        <v>0</v>
+      </c>
+      <c r="H93" t="inlineStr"/>
+      <c r="I93" t="n">
+        <v>0</v>
+      </c>
+      <c r="J93" t="n">
+        <v>0</v>
+      </c>
+      <c r="K93" t="n">
+        <v>1</v>
+      </c>
+      <c r="L93" t="n">
+        <v>0</v>
+      </c>
+      <c r="M93" t="inlineStr"/>
+      <c r="N93" t="inlineStr"/>
+      <c r="O93" t="n">
+        <v>0</v>
+      </c>
+      <c r="P93" t="inlineStr"/>
+      <c r="Q93" t="inlineStr"/>
+      <c r="R93" t="inlineStr">
+        <is>
+          <t>Orange Syrup</t>
+        </is>
+      </c>
+      <c r="S93" t="inlineStr"/>
+      <c r="T93" t="inlineStr"/>
+      <c r="U93" t="inlineStr"/>
+      <c r="V93" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="94">
+      <c r="A94" t="inlineStr">
+        <is>
+          <t>ZW02551</t>
+        </is>
+      </c>
+      <c r="B94" t="inlineStr">
+        <is>
+          <t>HQ Woburn</t>
+        </is>
+      </c>
+      <c r="C94" t="inlineStr">
+        <is>
+          <t>2026-07-01~2026-07-31</t>
+        </is>
+      </c>
+      <c r="D94" t="n">
+        <v>31</v>
+      </c>
+      <c r="E94" t="inlineStr">
+        <is>
+          <t>Passion Fruit Syrup</t>
+        </is>
+      </c>
+      <c r="F94" t="inlineStr">
+        <is>
+          <t>M34</t>
+        </is>
+      </c>
+      <c r="G94" t="n">
+        <v>0</v>
+      </c>
+      <c r="H94" t="inlineStr"/>
+      <c r="I94" t="n">
+        <v>0</v>
+      </c>
+      <c r="J94" t="n">
+        <v>0</v>
+      </c>
+      <c r="K94" t="n">
+        <v>1</v>
+      </c>
+      <c r="L94" t="n">
+        <v>0</v>
+      </c>
+      <c r="M94" t="inlineStr"/>
+      <c r="N94" t="inlineStr"/>
+      <c r="O94" t="n">
+        <v>0</v>
+      </c>
+      <c r="P94" t="inlineStr"/>
+      <c r="Q94" t="inlineStr"/>
+      <c r="R94" t="inlineStr">
+        <is>
+          <t>Passion Fruit Syrup</t>
+        </is>
+      </c>
+      <c r="S94" t="inlineStr"/>
+      <c r="T94" t="inlineStr"/>
+      <c r="U94" t="inlineStr"/>
+      <c r="V94" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="95">
+      <c r="A95" t="inlineStr">
+        <is>
+          <t>ZW02551</t>
+        </is>
+      </c>
+      <c r="B95" t="inlineStr">
+        <is>
+          <t>HQ Woburn</t>
+        </is>
+      </c>
+      <c r="C95" t="inlineStr">
+        <is>
+          <t>2026-07-01~2026-07-31</t>
+        </is>
+      </c>
+      <c r="D95" t="n">
+        <v>31</v>
+      </c>
+      <c r="E95" t="inlineStr">
+        <is>
+          <t>全脂牛奶 Whole Milk</t>
+        </is>
+      </c>
+      <c r="F95" t="inlineStr">
+        <is>
+          <t>M35</t>
+        </is>
+      </c>
+      <c r="G95" t="n">
+        <v>0</v>
+      </c>
+      <c r="H95" t="inlineStr"/>
+      <c r="I95" t="n">
+        <v>0</v>
+      </c>
+      <c r="J95" t="n">
+        <v>0</v>
+      </c>
+      <c r="K95" t="n">
+        <v>1</v>
+      </c>
+      <c r="L95" t="n">
+        <v>0</v>
+      </c>
+      <c r="M95" t="inlineStr"/>
+      <c r="N95" t="inlineStr"/>
+      <c r="O95" t="n">
+        <v>0</v>
+      </c>
+      <c r="P95" t="inlineStr"/>
+      <c r="Q95" t="inlineStr"/>
+      <c r="R95" t="inlineStr">
+        <is>
+          <t>Whole Milk</t>
+        </is>
+      </c>
+      <c r="S95" t="inlineStr"/>
+      <c r="T95" t="inlineStr"/>
+      <c r="U95" t="inlineStr"/>
+      <c r="V95" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="96">
+      <c r="A96" t="inlineStr">
+        <is>
+          <t>ZW02551</t>
+        </is>
+      </c>
+      <c r="B96" t="inlineStr">
+        <is>
+          <t>HQ Woburn</t>
+        </is>
+      </c>
+      <c r="C96" t="inlineStr">
+        <is>
+          <t>2026-07-01~2026-07-31</t>
+        </is>
+      </c>
+      <c r="D96" t="n">
+        <v>31</v>
+      </c>
+      <c r="E96" t="inlineStr">
+        <is>
+          <t>石榴糖浆 Pomegranate Syrup</t>
+        </is>
+      </c>
+      <c r="F96" t="inlineStr">
+        <is>
+          <t>MT14</t>
+        </is>
+      </c>
+      <c r="G96" t="n">
+        <v>0</v>
+      </c>
+      <c r="H96" t="inlineStr"/>
+      <c r="I96" t="n">
+        <v>0</v>
+      </c>
+      <c r="J96" t="n">
+        <v>0</v>
+      </c>
+      <c r="K96" t="n">
+        <v>1</v>
+      </c>
+      <c r="L96" t="n">
+        <v>0</v>
+      </c>
+      <c r="M96" t="inlineStr"/>
+      <c r="N96" t="inlineStr"/>
+      <c r="O96" t="n">
+        <v>0</v>
+      </c>
+      <c r="P96" t="inlineStr"/>
+      <c r="Q96" t="inlineStr"/>
+      <c r="R96" t="inlineStr">
+        <is>
+          <t>Pomegranate Syrup</t>
+        </is>
+      </c>
+      <c r="S96" t="inlineStr"/>
+      <c r="T96" t="inlineStr"/>
+      <c r="U96" t="inlineStr"/>
+      <c r="V96" t="n">
         <v>0</v>
       </c>
     </row>

</xml_diff>